<commit_message>
Update HOTUSDT.json at 2024-08-06_12-07-19 bestfile_scores 0.0012816329342791144 bestfile_sharp 0.0897616575121067
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="387">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1536,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU146"/>
+  <dimension ref="A1:CU147"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -41849,6 +41849,275 @@
       </c>
       <c r="CU146">
         <v>-0.6822914041817671</v>
+      </c>
+    </row>
+    <row r="147" spans="10:99">
+      <c r="J147" t="s">
+        <v>238</v>
+      </c>
+      <c r="K147">
+        <v>0.0009271508706103493</v>
+      </c>
+      <c r="L147">
+        <v>0.0009271508706103493</v>
+      </c>
+      <c r="M147">
+        <v>0.0003772496124334612</v>
+      </c>
+      <c r="N147">
+        <v>0.0003772496124334612</v>
+      </c>
+      <c r="O147">
+        <v>0.0007341407739547501</v>
+      </c>
+      <c r="P147">
+        <v>0.0007341407739547501</v>
+      </c>
+      <c r="Q147">
+        <v>0.000427802544585143</v>
+      </c>
+      <c r="R147">
+        <v>0.000427802544585143</v>
+      </c>
+      <c r="S147">
+        <v>5.186290271715415</v>
+      </c>
+      <c r="T147">
+        <v>4.126047943115981</v>
+      </c>
+      <c r="U147">
+        <v>0.9943079530884374</v>
+      </c>
+      <c r="V147">
+        <v>0.7441713851721259</v>
+      </c>
+      <c r="W147">
+        <v>0.08782631912769941</v>
+      </c>
+      <c r="X147">
+        <v>0.09612852812434385</v>
+      </c>
+      <c r="Y147">
+        <v>0.1487338338096725</v>
+      </c>
+      <c r="Z147">
+        <v>0.1765393432169604</v>
+      </c>
+      <c r="AA147">
+        <v>0.9979090421403467</v>
+      </c>
+      <c r="AB147">
+        <v>0.8631748366243617</v>
+      </c>
+      <c r="AC147">
+        <v>0.85245390722169</v>
+      </c>
+      <c r="AD147">
+        <v>0.9973853483851801</v>
+      </c>
+      <c r="AE147">
+        <v>0.8577699950051938</v>
+      </c>
+      <c r="AF147">
+        <v>0.8334553258441252</v>
+      </c>
+      <c r="AG147">
+        <v>0.009891723442382157</v>
+      </c>
+      <c r="AH147">
+        <v>0.01075541834616141</v>
+      </c>
+      <c r="AI147">
+        <v>0.9979090421403467</v>
+      </c>
+      <c r="AJ147">
+        <v>0.9973853483851801</v>
+      </c>
+      <c r="AK147">
+        <v>0.009891723442382157</v>
+      </c>
+      <c r="AL147">
+        <v>0.01075541834616141</v>
+      </c>
+      <c r="AM147" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN147">
+        <v>0.07466532002742356</v>
+      </c>
+      <c r="AO147">
+        <v>0.05158437131730968</v>
+      </c>
+      <c r="AP147">
+        <v>-559.644700872</v>
+      </c>
+      <c r="AQ147">
+        <v>-137.17975723</v>
+      </c>
+      <c r="AR147">
+        <v>27180.94354516747</v>
+      </c>
+      <c r="AS147">
+        <v>15022.66619276996</v>
+      </c>
+      <c r="AT147">
+        <v>25765.66907912802</v>
+      </c>
+      <c r="AU147">
+        <v>15022.66619276996</v>
+      </c>
+      <c r="AV147">
+        <v>1.718094354516747</v>
+      </c>
+      <c r="AW147">
+        <v>0.5022666192769965</v>
+      </c>
+      <c r="AX147">
+        <v>4.626705391718796</v>
+      </c>
+      <c r="AY147">
+        <v>5.805036321425896</v>
+      </c>
+      <c r="AZ147">
+        <v>83.15000000000001</v>
+      </c>
+      <c r="BA147">
+        <v>85.53333333333333</v>
+      </c>
+      <c r="BB147">
+        <v>0.06073549320104688</v>
+      </c>
+      <c r="BC147">
+        <v>0.1979569492821935</v>
+      </c>
+      <c r="BD147">
+        <v>-1147.156492128083</v>
+      </c>
+      <c r="BE147">
+        <v>-1273.531841107445</v>
+      </c>
+      <c r="BF147">
+        <v>2784</v>
+      </c>
+      <c r="BG147">
+        <v>2470</v>
+      </c>
+      <c r="BH147">
+        <v>1078.998611111111</v>
+      </c>
+      <c r="BI147">
+        <v>2812</v>
+      </c>
+      <c r="BJ147">
+        <v>1982</v>
+      </c>
+      <c r="BK147">
+        <v>5596</v>
+      </c>
+      <c r="BL147">
+        <v>4452</v>
+      </c>
+      <c r="BM147">
+        <v>0</v>
+      </c>
+      <c r="BN147">
+        <v>0</v>
+      </c>
+      <c r="BO147">
+        <v>95</v>
+      </c>
+      <c r="BP147">
+        <v>21</v>
+      </c>
+      <c r="BQ147">
+        <v>0</v>
+      </c>
+      <c r="BR147">
+        <v>0</v>
+      </c>
+      <c r="BS147">
+        <v>2689</v>
+      </c>
+      <c r="BT147">
+        <v>2449</v>
+      </c>
+      <c r="BU147">
+        <v>2812</v>
+      </c>
+      <c r="BV147">
+        <v>1982</v>
+      </c>
+      <c r="BW147">
+        <v>17180.94354516744</v>
+      </c>
+      <c r="BX147">
+        <v>5022.666192769993</v>
+      </c>
+      <c r="BY147">
+        <v>0.08872882728817136</v>
+      </c>
+      <c r="BZ147">
+        <v>0.2027142729554022</v>
+      </c>
+      <c r="CA147">
+        <v>0.1658107791868395</v>
+      </c>
+      <c r="CB147">
+        <v>0.3059584933131804</v>
+      </c>
+      <c r="CC147">
+        <v>0.01331063120855579</v>
+      </c>
+      <c r="CD147">
+        <v>0.0240731126461369</v>
+      </c>
+      <c r="CE147">
+        <v>0.01515624390504481</v>
+      </c>
+      <c r="CF147">
+        <v>0.03418969224219068</v>
+      </c>
+      <c r="CG147">
+        <v>17740.58824603944</v>
+      </c>
+      <c r="CH147">
+        <v>5159.845949999994</v>
+      </c>
+      <c r="CI147">
+        <v>18887.74473816753</v>
+      </c>
+      <c r="CJ147">
+        <v>6433.377791107439</v>
+      </c>
+      <c r="CK147">
+        <v>0.09383586056299457</v>
+      </c>
+      <c r="CL147">
+        <v>0.05546030914566657</v>
+      </c>
+      <c r="CM147">
+        <v>10000</v>
+      </c>
+      <c r="CO147">
+        <v>0.03147082673668765</v>
+      </c>
+      <c r="CP147">
+        <v>0.00459512684866973</v>
+      </c>
+      <c r="CQ147">
+        <v>9932751.742502673</v>
+      </c>
+      <c r="CR147">
+        <v>3613938.735498667</v>
+      </c>
+      <c r="CS147" s="2">
+        <v>45510.29086814423</v>
+      </c>
+      <c r="CT147">
+        <v>-0.7509273913693356</v>
+      </c>
+      <c r="CU147">
+        <v>-0.8707969045725891</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update IMXUSDT.json at 2024-08-06_15-18-22 bestfile_scores 0.0012231175625238234 bestfile_sharp 0.18265933800740458
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="388">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -743,6 +743,9 @@
   </si>
   <si>
     <t>HNTUSDT</t>
+  </si>
+  <si>
+    <t>HOTUSDT</t>
   </si>
   <si>
     <t>binance</t>
@@ -1536,7 +1539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU147"/>
+  <dimension ref="A1:CU148"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1951,7 +1954,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN2">
         <v>0.049606857</v>
@@ -2116,7 +2119,7 @@
         <v>0</v>
       </c>
       <c r="CS2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:99">
@@ -2232,7 +2235,7 @@
         <v>0</v>
       </c>
       <c r="AM3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN3">
         <v>0.04006526</v>
@@ -2397,7 +2400,7 @@
         <v>0</v>
       </c>
       <c r="CS3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" spans="1:99">
@@ -2513,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN4">
         <v>0.092575794</v>
@@ -2678,7 +2681,7 @@
         <v>0</v>
       </c>
       <c r="CS4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:99">
@@ -2794,7 +2797,7 @@
         <v>0</v>
       </c>
       <c r="AM5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN5">
         <v>0.027448502</v>
@@ -2959,7 +2962,7 @@
         <v>0</v>
       </c>
       <c r="CS5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:99">
@@ -3075,7 +3078,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN6">
         <v>0.083929868</v>
@@ -3240,7 +3243,7 @@
         <v>0</v>
       </c>
       <c r="CS6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:99">
@@ -3356,7 +3359,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN7">
         <v>0.145376251</v>
@@ -3521,7 +3524,7 @@
         <v>0</v>
       </c>
       <c r="CS7" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:99">
@@ -3637,7 +3640,7 @@
         <v>0</v>
       </c>
       <c r="AM8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN8">
         <v>0.087987204</v>
@@ -3802,7 +3805,7 @@
         <v>0</v>
       </c>
       <c r="CS8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:99">
@@ -3918,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="AM9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN9">
         <v>0.118237951</v>
@@ -4083,7 +4086,7 @@
         <v>0</v>
       </c>
       <c r="CS9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" spans="1:99">
@@ -4199,7 +4202,7 @@
         <v>0</v>
       </c>
       <c r="AM10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN10">
         <v>0.08106915200000001</v>
@@ -4364,7 +4367,7 @@
         <v>0</v>
       </c>
       <c r="CS10" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="11" spans="1:99">
@@ -4480,7 +4483,7 @@
         <v>0</v>
       </c>
       <c r="AM11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN11">
         <v>0.027960571</v>
@@ -4645,7 +4648,7 @@
         <v>0</v>
       </c>
       <c r="CS11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:99">
@@ -4761,7 +4764,7 @@
         <v>0</v>
       </c>
       <c r="AM12" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN12">
         <v>0.032951036</v>
@@ -4926,7 +4929,7 @@
         <v>0</v>
       </c>
       <c r="CS12" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:99">
@@ -5042,7 +5045,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN13">
         <v>0.179185242</v>
@@ -5207,7 +5210,7 @@
         <v>0</v>
       </c>
       <c r="CS13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:99">
@@ -5323,7 +5326,7 @@
         <v>0</v>
       </c>
       <c r="AM14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN14">
         <v>0.143233482</v>
@@ -5488,7 +5491,7 @@
         <v>0</v>
       </c>
       <c r="CS14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:99">
@@ -5604,7 +5607,7 @@
         <v>0</v>
       </c>
       <c r="AM15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN15">
         <v>0.138115134</v>
@@ -5769,7 +5772,7 @@
         <v>0</v>
       </c>
       <c r="CS15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:99">
@@ -5885,7 +5888,7 @@
         <v>0</v>
       </c>
       <c r="AM16" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN16">
         <v>0.09650975000000001</v>
@@ -6050,7 +6053,7 @@
         <v>0</v>
       </c>
       <c r="CS16" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:97">
@@ -6166,7 +6169,7 @@
         <v>0</v>
       </c>
       <c r="AM17" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN17">
         <v>0.060693695</v>
@@ -6331,7 +6334,7 @@
         <v>0</v>
       </c>
       <c r="CS17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:97">
@@ -6447,7 +6450,7 @@
         <v>0</v>
       </c>
       <c r="AM18" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN18">
         <v>0.107514363</v>
@@ -6612,7 +6615,7 @@
         <v>0</v>
       </c>
       <c r="CS18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:97">
@@ -6728,7 +6731,7 @@
         <v>0</v>
       </c>
       <c r="AM19" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN19">
         <v>0.014898256</v>
@@ -6893,7 +6896,7 @@
         <v>0</v>
       </c>
       <c r="CS19" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" spans="1:97">
@@ -7009,7 +7012,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN20">
         <v>0.02858403</v>
@@ -7174,7 +7177,7 @@
         <v>0</v>
       </c>
       <c r="CS20" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:97">
@@ -7290,7 +7293,7 @@
         <v>0</v>
       </c>
       <c r="AM21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN21">
         <v>0.082273481</v>
@@ -7455,7 +7458,7 @@
         <v>0</v>
       </c>
       <c r="CS21" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" spans="1:97">
@@ -7571,7 +7574,7 @@
         <v>0</v>
       </c>
       <c r="AM22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN22">
         <v>0.012592558</v>
@@ -7736,7 +7739,7 @@
         <v>0</v>
       </c>
       <c r="CS22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:97">
@@ -7852,7 +7855,7 @@
         <v>0</v>
       </c>
       <c r="AM23" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN23">
         <v>0.00903967</v>
@@ -8017,7 +8020,7 @@
         <v>0</v>
       </c>
       <c r="CS23" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="24" spans="1:97">
@@ -8133,7 +8136,7 @@
         <v>0</v>
       </c>
       <c r="AM24" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN24">
         <v>0.030046089</v>
@@ -8298,7 +8301,7 @@
         <v>0</v>
       </c>
       <c r="CS24" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:97">
@@ -8414,7 +8417,7 @@
         <v>0</v>
       </c>
       <c r="AM25" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN25">
         <v>0.010607012</v>
@@ -8579,7 +8582,7 @@
         <v>0</v>
       </c>
       <c r="CS25" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:97">
@@ -8695,7 +8698,7 @@
         <v>0</v>
       </c>
       <c r="AM26" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN26">
         <v>0.053096335</v>
@@ -8860,7 +8863,7 @@
         <v>0</v>
       </c>
       <c r="CS26" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27" spans="1:97">
@@ -8976,7 +8979,7 @@
         <v>0</v>
       </c>
       <c r="AM27" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN27">
         <v>0.092674047</v>
@@ -9141,7 +9144,7 @@
         <v>0</v>
       </c>
       <c r="CS27" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:97">
@@ -9257,7 +9260,7 @@
         <v>0</v>
       </c>
       <c r="AM28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN28">
         <v>0.03099706</v>
@@ -9422,7 +9425,7 @@
         <v>0</v>
       </c>
       <c r="CS28" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" spans="1:97">
@@ -9538,7 +9541,7 @@
         <v>0</v>
       </c>
       <c r="AM29" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN29">
         <v>0.069423731</v>
@@ -9703,7 +9706,7 @@
         <v>0</v>
       </c>
       <c r="CS29" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" spans="1:97">
@@ -9819,7 +9822,7 @@
         <v>0</v>
       </c>
       <c r="AM30" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN30">
         <v>0.060424834</v>
@@ -9984,7 +9987,7 @@
         <v>0</v>
       </c>
       <c r="CS30" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:97">
@@ -10100,7 +10103,7 @@
         <v>0</v>
       </c>
       <c r="AM31" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN31">
         <v>0.056666776</v>
@@ -10265,7 +10268,7 @@
         <v>0</v>
       </c>
       <c r="CS31" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:97">
@@ -10381,7 +10384,7 @@
         <v>0</v>
       </c>
       <c r="AM32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN32">
         <v>0.098888062</v>
@@ -10546,7 +10549,7 @@
         <v>0</v>
       </c>
       <c r="CS32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="33" spans="1:99">
@@ -10662,7 +10665,7 @@
         <v>0</v>
       </c>
       <c r="AM33" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN33">
         <v>0.035815903</v>
@@ -10827,7 +10830,7 @@
         <v>0</v>
       </c>
       <c r="CS33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="34" spans="1:99">
@@ -10943,7 +10946,7 @@
         <v>0</v>
       </c>
       <c r="AM34" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN34">
         <v>0.037311133</v>
@@ -11108,7 +11111,7 @@
         <v>0</v>
       </c>
       <c r="CS34" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="CT34">
         <v>-0.814742818</v>
@@ -11230,7 +11233,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN35">
         <v>0.041330496</v>
@@ -11395,7 +11398,7 @@
         <v>0</v>
       </c>
       <c r="CS35" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="CT35">
         <v>-0.753066891</v>
@@ -11517,7 +11520,7 @@
         <v>0</v>
       </c>
       <c r="AM36" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN36">
         <v>0.047772102</v>
@@ -11682,7 +11685,7 @@
         <v>0</v>
       </c>
       <c r="CS36" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="CT36">
         <v>-0.872335259</v>
@@ -11804,7 +11807,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN37">
         <v>0.060484521</v>
@@ -11969,7 +11972,7 @@
         <v>0</v>
       </c>
       <c r="CS37" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="CT37">
         <v>-0.759885442</v>
@@ -12091,7 +12094,7 @@
         <v>0</v>
       </c>
       <c r="AM38" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN38">
         <v>0.061007062</v>
@@ -12256,7 +12259,7 @@
         <v>0</v>
       </c>
       <c r="CS38" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="CT38">
         <v>-0.838900609</v>
@@ -12378,7 +12381,7 @@
         <v>0</v>
       </c>
       <c r="AM39" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN39">
         <v>0.025236369</v>
@@ -12543,7 +12546,7 @@
         <v>0</v>
       </c>
       <c r="CS39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="CT39">
         <v>-0.780218664</v>
@@ -12665,7 +12668,7 @@
         <v>0</v>
       </c>
       <c r="AM40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN40">
         <v>0.031804424</v>
@@ -12830,7 +12833,7 @@
         <v>0</v>
       </c>
       <c r="CS40" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="CT40">
         <v>-0.79992089</v>
@@ -12952,7 +12955,7 @@
         <v>0</v>
       </c>
       <c r="AM41" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN41">
         <v>0.072404657</v>
@@ -13117,7 +13120,7 @@
         <v>0</v>
       </c>
       <c r="CS41" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="CT41">
         <v>-0.528089775</v>
@@ -13239,7 +13242,7 @@
         <v>0</v>
       </c>
       <c r="AM42" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN42">
         <v>0.06821192299999999</v>
@@ -13404,7 +13407,7 @@
         <v>0</v>
       </c>
       <c r="CS42" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="CT42">
         <v>-0.754849911</v>
@@ -13526,7 +13529,7 @@
         <v>0</v>
       </c>
       <c r="AM43" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN43">
         <v>0.069326524</v>
@@ -13691,7 +13694,7 @@
         <v>0</v>
       </c>
       <c r="CS43" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="CT43">
         <v>-0.7655395739999999</v>
@@ -13813,7 +13816,7 @@
         <v>0</v>
       </c>
       <c r="AM44" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN44">
         <v>0.036991009</v>
@@ -13978,7 +13981,7 @@
         <v>0</v>
       </c>
       <c r="CS44" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="CT44">
         <v>-0.829764531</v>
@@ -14100,7 +14103,7 @@
         <v>0</v>
       </c>
       <c r="AM45" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN45">
         <v>0.036729519</v>
@@ -14265,7 +14268,7 @@
         <v>0</v>
       </c>
       <c r="CS45" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="CT45">
         <v>-0.404237806</v>
@@ -14387,7 +14390,7 @@
         <v>0</v>
       </c>
       <c r="AM46" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN46">
         <v>0.045071814</v>
@@ -14552,7 +14555,7 @@
         <v>0</v>
       </c>
       <c r="CS46" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="CT46">
         <v>-0.703677808</v>
@@ -14674,7 +14677,7 @@
         <v>0</v>
       </c>
       <c r="AM47" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN47">
         <v>0.0580535</v>
@@ -14839,7 +14842,7 @@
         <v>0</v>
       </c>
       <c r="CS47" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="CT47">
         <v>-0.753715321</v>
@@ -14961,7 +14964,7 @@
         <v>0</v>
       </c>
       <c r="AM48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN48">
         <v>0.056639031</v>
@@ -15126,7 +15129,7 @@
         <v>0</v>
       </c>
       <c r="CS48" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="CT48">
         <v>-0.71793867</v>
@@ -15248,7 +15251,7 @@
         <v>0</v>
       </c>
       <c r="AM49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN49">
         <v>0.074241638</v>
@@ -15413,7 +15416,7 @@
         <v>0</v>
       </c>
       <c r="CS49" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="CT49">
         <v>-0.655169358</v>
@@ -15535,7 +15538,7 @@
         <v>0</v>
       </c>
       <c r="AM50" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN50">
         <v>0.05430774</v>
@@ -15700,7 +15703,7 @@
         <v>0</v>
       </c>
       <c r="CS50" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="CT50">
         <v>-0.6872439380000001</v>
@@ -15822,7 +15825,7 @@
         <v>0</v>
       </c>
       <c r="AM51" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN51">
         <v>0.080539377</v>
@@ -15987,7 +15990,7 @@
         <v>0</v>
       </c>
       <c r="CS51" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="CT51">
         <v>-0.596275172</v>
@@ -16109,7 +16112,7 @@
         <v>0</v>
       </c>
       <c r="AM52" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN52">
         <v>0.032588051</v>
@@ -16274,7 +16277,7 @@
         <v>0</v>
       </c>
       <c r="CS52" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="CT52">
         <v>-0.808081961</v>
@@ -16396,7 +16399,7 @@
         <v>0</v>
       </c>
       <c r="AM53" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN53">
         <v>0.026475554</v>
@@ -16561,7 +16564,7 @@
         <v>0</v>
       </c>
       <c r="CS53" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CT53">
         <v>-0.77227813</v>
@@ -16683,7 +16686,7 @@
         <v>0</v>
       </c>
       <c r="AM54" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN54">
         <v>0.0245106310926154</v>
@@ -16848,7 +16851,7 @@
         <v>0</v>
       </c>
       <c r="CS54" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="CT54">
         <v>-0.8664117478627688</v>
@@ -16967,7 +16970,7 @@
         <v>0</v>
       </c>
       <c r="AM55" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN55">
         <v>0.0779439577559576</v>
@@ -17132,7 +17135,7 @@
         <v>0</v>
       </c>
       <c r="CS55" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="CT55">
         <v>-0.7108907987632488</v>
@@ -17248,7 +17251,7 @@
         <v>0</v>
       </c>
       <c r="AM56" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN56">
         <v>0.0402740604837066</v>
@@ -17413,7 +17416,7 @@
         <v>0</v>
       </c>
       <c r="CS56" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="CT56">
         <v>-0.7447372903525753</v>
@@ -17526,7 +17529,7 @@
         <v>0</v>
       </c>
       <c r="AM57" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN57">
         <v>0.0441363962743036</v>
@@ -17691,7 +17694,7 @@
         <v>0</v>
       </c>
       <c r="CS57" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="CT57">
         <v>-0.7777179486581601</v>
@@ -17804,7 +17807,7 @@
         <v>0</v>
       </c>
       <c r="AM58" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN58">
         <v>0.0589646348207879</v>
@@ -17969,7 +17972,7 @@
         <v>0</v>
       </c>
       <c r="CS58" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="CT58">
         <v>-0.7757098341832183</v>
@@ -18082,7 +18085,7 @@
         <v>0</v>
       </c>
       <c r="AM59" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN59">
         <v>0.0088498418945465</v>
@@ -18247,7 +18250,7 @@
         <v>0</v>
       </c>
       <c r="CS59" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="CT59">
         <v>-0.9614802262041642</v>
@@ -18360,7 +18363,7 @@
         <v>0</v>
       </c>
       <c r="AM60" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN60">
         <v>0.0438527807624406</v>
@@ -18525,7 +18528,7 @@
         <v>0</v>
       </c>
       <c r="CS60" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="CT60">
         <v>-0.6569921650581255</v>
@@ -18638,7 +18641,7 @@
         <v>0</v>
       </c>
       <c r="AM61" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN61">
         <v>0.0175722673111926</v>
@@ -18803,7 +18806,7 @@
         <v>0</v>
       </c>
       <c r="CS61" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="CT61">
         <v>-0.924044412704054</v>
@@ -18916,7 +18919,7 @@
         <v>0</v>
       </c>
       <c r="AM62" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN62">
         <v>0.0551224625318549</v>
@@ -19081,7 +19084,7 @@
         <v>0</v>
       </c>
       <c r="CS62" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="CT62">
         <v>-0.6213262971882773</v>
@@ -19194,7 +19197,7 @@
         <v>0</v>
       </c>
       <c r="AM63" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN63">
         <v>0.0157574961492794</v>
@@ -19359,7 +19362,7 @@
         <v>0</v>
       </c>
       <c r="CS63" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="CT63">
         <v>-0.9477002142299265</v>
@@ -19472,7 +19475,7 @@
         <v>0</v>
       </c>
       <c r="AM64" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN64">
         <v>0.0348775184726272</v>
@@ -19637,7 +19640,7 @@
         <v>0</v>
       </c>
       <c r="CS64" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="CT64">
         <v>-0.7774025388699596</v>
@@ -19750,7 +19753,7 @@
         <v>0</v>
       </c>
       <c r="AM65" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN65">
         <v>0.0617007650932976</v>
@@ -19915,7 +19918,7 @@
         <v>0</v>
       </c>
       <c r="CS65" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="CT65">
         <v>-0.8140402180385446</v>
@@ -20028,7 +20031,7 @@
         <v>0.0108330657640134</v>
       </c>
       <c r="AM66" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN66">
         <v>0.0122896465671382</v>
@@ -20199,7 +20202,7 @@
         <v>28802806.1197283</v>
       </c>
       <c r="CS66" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="CT66">
         <v>-0.7661604887809055</v>
@@ -20312,7 +20315,7 @@
         <v>0.009662114019183699</v>
       </c>
       <c r="AM67" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN67">
         <v>0.0157075521173083</v>
@@ -20483,7 +20486,7 @@
         <v>12816652.38654842</v>
       </c>
       <c r="CS67" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="CT67">
         <v>-0.843107865610227</v>
@@ -20596,7 +20599,7 @@
         <v>0.009682496602030599</v>
       </c>
       <c r="AM68" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN68">
         <v>0.019453807476403</v>
@@ -20767,7 +20770,7 @@
         <v>362119.31393403</v>
       </c>
       <c r="CS68" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="CT68">
         <v>-0.7040504011377985</v>
@@ -20880,7 +20883,7 @@
         <v>0.009502809785555901</v>
       </c>
       <c r="AM69" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN69">
         <v>0.0467996269477206</v>
@@ -21051,7 +21054,7 @@
         <v>3444392.687119505</v>
       </c>
       <c r="CS69" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="CT69">
         <v>-0.5814104972412503</v>
@@ -21161,7 +21164,7 @@
         <v>0.0100375716524098</v>
       </c>
       <c r="AM70" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN70">
         <v>0.0260012684361012</v>
@@ -21332,7 +21335,7 @@
         <v>8020410.490554446</v>
       </c>
       <c r="CS70" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="CT70">
         <v>-0.1225754953154068</v>
@@ -21439,7 +21442,7 @@
         <v>0.0030270679524292</v>
       </c>
       <c r="AM71" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN71">
         <v>0.007629803458883</v>
@@ -21610,7 +21613,7 @@
         <v>6690404.196816532</v>
       </c>
       <c r="CS71" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="CT71">
         <v>-0.943556327266077</v>
@@ -21714,7 +21717,7 @@
         <v>0.0071318120684325</v>
       </c>
       <c r="AM72" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN72">
         <v>0.0106438024257861</v>
@@ -21885,7 +21888,7 @@
         <v>2333580.086114224</v>
       </c>
       <c r="CS72" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="CT72">
         <v>-0.9017649135974464</v>
@@ -21989,7 +21992,7 @@
         <v>0.008671749707596699</v>
       </c>
       <c r="AM73" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN73">
         <v>0.008922434565822699</v>
@@ -22160,7 +22163,7 @@
         <v>4050354.030474017</v>
       </c>
       <c r="CS73" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="CT73">
         <v>-0.9011542748767548</v>
@@ -22264,7 +22267,7 @@
         <v>0.0061287699408089</v>
       </c>
       <c r="AM74" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN74">
         <v>0.0100444206462455</v>
@@ -22435,7 +22438,7 @@
         <v>284228.7150822567</v>
       </c>
       <c r="CS74" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="CT74">
         <v>-0.9022640234515124</v>
@@ -22539,7 +22542,7 @@
         <v>0.009112086818146899</v>
       </c>
       <c r="AM75" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN75">
         <v>0.0105885988628848</v>
@@ -22710,7 +22713,7 @@
         <v>9238253.926865038</v>
       </c>
       <c r="CS75" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="CT75">
         <v>-0.8442464713130005</v>
@@ -22814,7 +22817,7 @@
         <v>0.0120332146147572</v>
       </c>
       <c r="AM76" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN76">
         <v>0.005689041712621</v>
@@ -22985,7 +22988,7 @@
         <v>103761437.1558867</v>
       </c>
       <c r="CS76" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="CT76">
         <v>-0.9172425776350784</v>
@@ -23089,7 +23092,7 @@
         <v>0.009980777925547499</v>
       </c>
       <c r="AM77" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN77">
         <v>0.0213191472253163</v>
@@ -23260,7 +23263,7 @@
         <v>11075597.03060125</v>
       </c>
       <c r="CS77" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="CT77">
         <v>-0.7048134977852135</v>
@@ -23361,7 +23364,7 @@
         <v>0.008640349693688199</v>
       </c>
       <c r="AM78" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN78">
         <v>0.0310379691662141</v>
@@ -23532,7 +23535,7 @@
         <v>4941591.885046311</v>
       </c>
       <c r="CS78" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="CT78">
         <v>-0.6921566954508142</v>
@@ -23633,7 +23636,7 @@
         <v>0.0052151469726826</v>
       </c>
       <c r="AM79" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN79">
         <v>0.0187749711217366</v>
@@ -23804,7 +23807,7 @@
         <v>13794144.77050867</v>
       </c>
       <c r="CS79" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="CT79">
         <v>-0.6546270123512354</v>
@@ -23905,7 +23908,7 @@
         <v>0.0083235819058295</v>
       </c>
       <c r="AM80" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN80">
         <v>0.0531066176371749</v>
@@ -24076,7 +24079,7 @@
         <v>1271425.087705649</v>
       </c>
       <c r="CS80" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="CT80">
         <v>-0.3384511866527668</v>
@@ -24177,7 +24180,7 @@
         <v>0.0041067346844988</v>
       </c>
       <c r="AM81" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN81">
         <v>0.0376358519870464</v>
@@ -24348,7 +24351,7 @@
         <v>8472790.733285822</v>
       </c>
       <c r="CS81" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="CT81">
         <v>-0.5869016106017596</v>
@@ -24449,7 +24452,7 @@
         <v>0.0055266741344329</v>
       </c>
       <c r="AM82" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN82">
         <v>0.0047447694558675</v>
@@ -24620,7 +24623,7 @@
         <v>6299784.652790904</v>
       </c>
       <c r="CS82" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="CT82">
         <v>-0.9571664073286058</v>
@@ -24721,7 +24724,7 @@
         <v>0.0083610158619657</v>
       </c>
       <c r="AM83" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN83">
         <v>0.0075895877096284</v>
@@ -24892,7 +24895,7 @@
         <v>9553962.229671104</v>
       </c>
       <c r="CS83" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="CT83">
         <v>-0.7975627900619038</v>
@@ -24993,7 +24996,7 @@
         <v>0.0110102665992773</v>
       </c>
       <c r="AM84" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN84">
         <v>0.0289129415567337</v>
@@ -25164,7 +25167,7 @@
         <v>9017755.465507764</v>
       </c>
       <c r="CS84" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="CT84">
         <v>-0.641321453686593</v>
@@ -25262,7 +25265,7 @@
         <v>0.001235474151197</v>
       </c>
       <c r="AM85" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN85">
         <v>0.0236860634403801</v>
@@ -25433,7 +25436,7 @@
         <v>395804.1998002621</v>
       </c>
       <c r="CS85" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="CT85">
         <v>-0.8468525619890503</v>
@@ -25531,7 +25534,7 @@
         <v>0.0069339646256509</v>
       </c>
       <c r="AM86" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN86">
         <v>0.0046798420774097</v>
@@ -25702,7 +25705,7 @@
         <v>5470308.140646266</v>
       </c>
       <c r="CS86" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="CT86">
         <v>-0.9414869172232342</v>
@@ -25800,7 +25803,7 @@
         <v>0.0084303895709902</v>
       </c>
       <c r="AM87" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN87">
         <v>0.0220548762227611</v>
@@ -25971,7 +25974,7 @@
         <v>10570112.91971009</v>
       </c>
       <c r="CS87" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="CT87">
         <v>-0.8207903291654746</v>
@@ -26069,7 +26072,7 @@
         <v>0.0046858616922062</v>
       </c>
       <c r="AM88" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN88">
         <v>0.0514935425696241</v>
@@ -26240,7 +26243,7 @@
         <v>5725644.496349121</v>
       </c>
       <c r="CS88" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="CT88">
         <v>-0.561712415905279</v>
@@ -26338,7 +26341,7 @@
         <v>0.0039939215766598</v>
       </c>
       <c r="AM89" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN89">
         <v>0.012222058764571</v>
@@ -26509,7 +26512,7 @@
         <v>1429804.32644608</v>
       </c>
       <c r="CS89" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="CT89">
         <v>-0.9176379634509604</v>
@@ -26607,7 +26610,7 @@
         <v>0.0042088758977745</v>
       </c>
       <c r="AM90" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN90">
         <v>0.019939030911244</v>
@@ -26778,7 +26781,7 @@
         <v>4722406.067514317</v>
       </c>
       <c r="CS90" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="CT90">
         <v>-0.9278452363120948</v>
@@ -26876,7 +26879,7 @@
         <v>0.0090603002679094</v>
       </c>
       <c r="AM91" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN91">
         <v>0.0130335524359802</v>
@@ -27047,7 +27050,7 @@
         <v>2899232.912138085</v>
       </c>
       <c r="CS91" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="CT91">
         <v>-0.8179686291978085</v>
@@ -27145,7 +27148,7 @@
         <v>0.0034278853232647</v>
       </c>
       <c r="AM92" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN92">
         <v>0.0267226315229668</v>
@@ -27316,7 +27319,7 @@
         <v>1448171.53934798</v>
       </c>
       <c r="CS92" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="CT92">
         <v>-0.8215150584575165</v>
@@ -27414,7 +27417,7 @@
         <v>0.0078801601208179</v>
       </c>
       <c r="AM93" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN93">
         <v>0.0221393128933173</v>
@@ -27585,7 +27588,7 @@
         <v>16635452.15900955</v>
       </c>
       <c r="CS93" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="CT93">
         <v>-0.7542388832888753</v>
@@ -27683,7 +27686,7 @@
         <v>0.0148358454007108</v>
       </c>
       <c r="AM94" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN94">
         <v>0.0142895129437342</v>
@@ -27854,7 +27857,7 @@
         <v>118847.66881</v>
       </c>
       <c r="CS94" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="CT94">
         <v>-0.8706219162560768</v>
@@ -27952,7 +27955,7 @@
         <v>0.00777307269066</v>
       </c>
       <c r="AM95" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN95">
         <v>0.028345432375321</v>
@@ -28123,7 +28126,7 @@
         <v>9989976.067409206</v>
       </c>
       <c r="CS95" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="CT95">
         <v>-0.7702665229627835</v>
@@ -28221,7 +28224,7 @@
         <v>0.005069566938105</v>
       </c>
       <c r="AM96" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN96">
         <v>0.0378882038525435</v>
@@ -28392,7 +28395,7 @@
         <v>4195010.116009732</v>
       </c>
       <c r="CS96" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="CT96">
         <v>-0.6208027078099908</v>
@@ -28490,7 +28493,7 @@
         <v>0.0109181034800677</v>
       </c>
       <c r="AM97" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN97">
         <v>0.0464479162381462</v>
@@ -28661,7 +28664,7 @@
         <v>1753546.300271091</v>
       </c>
       <c r="CS97" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="CT97">
         <v>-0.6637406607330143</v>
@@ -28759,7 +28762,7 @@
         <v>0.0073561352130028</v>
       </c>
       <c r="AM98" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN98">
         <v>0.0129973328606765</v>
@@ -28930,7 +28933,7 @@
         <v>8525723.260530123</v>
       </c>
       <c r="CS98" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="CT98">
         <v>-0.6066396906320848</v>
@@ -29028,7 +29031,7 @@
         <v>0.0010483764611907</v>
       </c>
       <c r="AM99" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN99">
         <v>0.0224095392580651</v>
@@ -29199,7 +29202,7 @@
         <v>555000.5818001842</v>
       </c>
       <c r="CS99" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="CT99">
         <v>-0.7930559623825889</v>
@@ -29297,7 +29300,7 @@
         <v>0.0034227206580065</v>
       </c>
       <c r="AM100" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN100">
         <v>0.0120356538583077</v>
@@ -29468,7 +29471,7 @@
         <v>8829982.660321526</v>
       </c>
       <c r="CS100" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="CT100">
         <v>-0.8625963918106255</v>
@@ -29566,7 +29569,7 @@
         <v>0.0024512168149686</v>
       </c>
       <c r="AM101" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN101">
         <v>0.0237148028402029</v>
@@ -29737,7 +29740,7 @@
         <v>3109464.939265249</v>
       </c>
       <c r="CS101" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="CT101">
         <v>-0.8320151516141147</v>
@@ -29835,7 +29838,7 @@
         <v>0.0013136523187938</v>
       </c>
       <c r="AM102" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN102">
         <v>0.0039597254802618</v>
@@ -30006,7 +30009,7 @@
         <v>1199182.410839436</v>
       </c>
       <c r="CS102" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="CT102">
         <v>-0.9034091343725908</v>
@@ -30104,7 +30107,7 @@
         <v>0.0026660229792492</v>
       </c>
       <c r="AM103" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN103">
         <v>0.0062754689148565</v>
@@ -30275,7 +30278,7 @@
         <v>5608278.16173986</v>
       </c>
       <c r="CS103" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="CT103">
         <v>-0.8495964311677586</v>
@@ -30373,7 +30376,7 @@
         <v>0.0095889911638783</v>
       </c>
       <c r="AM104" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN104">
         <v>0.0276610340172863</v>
@@ -30544,7 +30547,7 @@
         <v>16198187.75410762</v>
       </c>
       <c r="CS104" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="CT104">
         <v>-0.8581350323980486</v>
@@ -30642,7 +30645,7 @@
         <v>0.0090102837599302</v>
       </c>
       <c r="AM105" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN105">
         <v>0.0216087690726687</v>
@@ -30813,7 +30816,7 @@
         <v>10577375.81046865</v>
       </c>
       <c r="CS105" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="CT105">
         <v>-0.8842562871250494</v>
@@ -30911,7 +30914,7 @@
         <v>0.0050995967216395</v>
       </c>
       <c r="AM106" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN106">
         <v>0.0064663828879011</v>
@@ -31082,7 +31085,7 @@
         <v>8161103.390277231</v>
       </c>
       <c r="CS106" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="CT106">
         <v>-0.8751724322696175</v>
@@ -31180,7 +31183,7 @@
         <v>0.008368149950938699</v>
       </c>
       <c r="AM107" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN107">
         <v>0.0044562593205472</v>
@@ -31351,7 +31354,7 @@
         <v>8562542.046147738</v>
       </c>
       <c r="CS107" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="CT107">
         <v>-0.9169005340500024</v>
@@ -31449,7 +31452,7 @@
         <v>0.0065618399294816</v>
       </c>
       <c r="AM108" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN108">
         <v>0.0115970759513037</v>
@@ -31620,7 +31623,7 @@
         <v>5094802.189709073</v>
       </c>
       <c r="CS108" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="CT108">
         <v>-0.807087633056609</v>
@@ -31718,7 +31721,7 @@
         <v>0.0039283848188842</v>
       </c>
       <c r="AM109" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN109">
         <v>0.0506122383924143</v>
@@ -31889,7 +31892,7 @@
         <v>2688942.923710383</v>
       </c>
       <c r="CS109" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="CT109">
         <v>-0.6156032480827009</v>
@@ -31987,7 +31990,7 @@
         <v>0.0110575018573894</v>
       </c>
       <c r="AM110" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN110">
         <v>0.0182408073926103</v>
@@ -32158,7 +32161,7 @@
         <v>7113237.577421894</v>
       </c>
       <c r="CS110" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="CT110">
         <v>-0.7629790982692873</v>
@@ -32256,7 +32259,7 @@
         <v>0.0079211631943229</v>
       </c>
       <c r="AM111" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN111">
         <v>0.0160665598628607</v>
@@ -32427,7 +32430,7 @@
         <v>7296357.590261763</v>
       </c>
       <c r="CS111" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="CT111">
         <v>-0.8942723506201351</v>
@@ -32525,7 +32528,7 @@
         <v>0.0045682228774332</v>
       </c>
       <c r="AM112" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN112">
         <v>0.037886406926907</v>
@@ -32696,7 +32699,7 @@
         <v>646350.5069878154</v>
       </c>
       <c r="CS112" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="CT112">
         <v>-0.0916621825765546</v>
@@ -32794,7 +32797,7 @@
         <v>0.0103540243512939</v>
       </c>
       <c r="AM113" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN113">
         <v>0.0123420077084287</v>
@@ -32965,7 +32968,7 @@
         <v>16980708.42353759</v>
       </c>
       <c r="CS113" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="CT113">
         <v>-0.8006705745635164</v>
@@ -33063,7 +33066,7 @@
         <v>0.0064839021721033</v>
       </c>
       <c r="AM114" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN114">
         <v>0.0163921516174475</v>
@@ -33234,7 +33237,7 @@
         <v>778558.4127862654</v>
       </c>
       <c r="CS114" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="CT114">
         <v>-0.7935423347142916</v>
@@ -33332,7 +33335,7 @@
         <v>0.0115121978063762</v>
       </c>
       <c r="AM115" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN115">
         <v>0.0122833373375532</v>
@@ -33503,7 +33506,7 @@
         <v>22312718.74654885</v>
       </c>
       <c r="CS115" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="CT115">
         <v>-0.833943178203995</v>
@@ -33601,7 +33604,7 @@
         <v>0.0085575638145724</v>
       </c>
       <c r="AM116" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN116">
         <v>0.0253654749054445</v>
@@ -33772,7 +33775,7 @@
         <v>55051148.20247716</v>
       </c>
       <c r="CS116" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="CT116">
         <v>-0.7450076808546802</v>
@@ -33870,7 +33873,7 @@
         <v>0.0073550550024841</v>
       </c>
       <c r="AM117" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN117">
         <v>0.0189839179655455</v>
@@ -34041,7 +34044,7 @@
         <v>7593228.666961946</v>
       </c>
       <c r="CS117" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="CT117">
         <v>-0.5920454049159357</v>
@@ -34139,7 +34142,7 @@
         <v>0.0080994776472478</v>
       </c>
       <c r="AM118" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN118">
         <v>0.0067043103411634</v>
@@ -34310,7 +34313,7 @@
         <v>8613700.914603613</v>
       </c>
       <c r="CS118" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="CT118">
         <v>-0.9326775287918464</v>
@@ -34408,7 +34411,7 @@
         <v>0.0068550971234694</v>
       </c>
       <c r="AM119" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN119">
         <v>0.009392776226783601</v>
@@ -34579,7 +34582,7 @@
         <v>2380328.733367264</v>
       </c>
       <c r="CS119" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="CT119">
         <v>-0.955941339278515</v>
@@ -34677,7 +34680,7 @@
         <v>0.0038610240640448</v>
       </c>
       <c r="AM120" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN120">
         <v>0.0077083561528932</v>
@@ -34848,7 +34851,7 @@
         <v>872704.4135421006</v>
       </c>
       <c r="CS120" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="CT120">
         <v>-0.8980421674690441</v>
@@ -34946,7 +34949,7 @@
         <v>0.007825344507997999</v>
       </c>
       <c r="AM121" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN121">
         <v>0.0327708854210512</v>
@@ -35117,7 +35120,7 @@
         <v>10271258.08902804</v>
       </c>
       <c r="CS121" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="CT121">
         <v>-0.7644558396778582</v>
@@ -35215,7 +35218,7 @@
         <v>0.0053863780237919</v>
       </c>
       <c r="AM122" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN122">
         <v>0.0318217118436193</v>
@@ -35386,7 +35389,7 @@
         <v>4219262.028734344</v>
       </c>
       <c r="CS122" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="CT122">
         <v>-0.7390744315992817</v>
@@ -35484,7 +35487,7 @@
         <v>0.008317099460099901</v>
       </c>
       <c r="AM123" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN123">
         <v>0.0412544366764669</v>
@@ -35655,7 +35658,7 @@
         <v>7884481.26725769</v>
       </c>
       <c r="CS123" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="CT123">
         <v>-0.7831546722232047</v>
@@ -35753,7 +35756,7 @@
         <v>0.0032418393755305</v>
       </c>
       <c r="AM124" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN124">
         <v>0.0499292345312228</v>
@@ -35924,7 +35927,7 @@
         <v>4199685.074142367</v>
       </c>
       <c r="CS124" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="CT124">
         <v>-0.7053510752114568</v>
@@ -36022,7 +36025,7 @@
         <v>0.0105307693727994</v>
       </c>
       <c r="AM125" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN125">
         <v>0.0209369586410007</v>
@@ -36193,7 +36196,7 @@
         <v>14590537.25038491</v>
       </c>
       <c r="CS125" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="CT125">
         <v>-0.7252315072660098</v>
@@ -36291,7 +36294,7 @@
         <v>0.0051130877078413</v>
       </c>
       <c r="AM126" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN126">
         <v>0.0123868401976321</v>
@@ -36462,7 +36465,7 @@
         <v>716228.3326648935</v>
       </c>
       <c r="CS126" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="CT126">
         <v>-0.892232561911074</v>
@@ -36560,7 +36563,7 @@
         <v>0.0103267254619839</v>
       </c>
       <c r="AM127" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN127">
         <v>0.0276741525944277</v>
@@ -36731,7 +36734,7 @@
         <v>7960049.437302528</v>
       </c>
       <c r="CS127" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="CT127">
         <v>-0.7368411844597273</v>
@@ -36829,7 +36832,7 @@
         <v>0.001129927884937</v>
       </c>
       <c r="AM128" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN128">
         <v>0.0069498164483821</v>
@@ -37000,7 +37003,7 @@
         <v>1259981.153790825</v>
       </c>
       <c r="CS128" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="CT128">
         <v>-0.9143802706411296</v>
@@ -37098,7 +37101,7 @@
         <v>0.0097288328816258</v>
       </c>
       <c r="AM129" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN129">
         <v>0.0275626982729415</v>
@@ -37269,7 +37272,7 @@
         <v>16803825.65057263</v>
       </c>
       <c r="CS129" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="CT129">
         <v>-0.8590793790924167</v>
@@ -37367,7 +37370,7 @@
         <v>0.0115638527937927</v>
       </c>
       <c r="AM130" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN130">
         <v>0.009514899377222301</v>
@@ -37538,7 +37541,7 @@
         <v>7461415.917733567</v>
       </c>
       <c r="CS130" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="CT130">
         <v>-0.7834455371012616</v>
@@ -37636,7 +37639,7 @@
         <v>0.0066617897392062</v>
       </c>
       <c r="AM131" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN131">
         <v>0.0175240810959318</v>
@@ -37807,7 +37810,7 @@
         <v>1295517.443775632</v>
       </c>
       <c r="CS131" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="CT131">
         <v>-0.7832286955751367</v>
@@ -37905,7 +37908,7 @@
         <v>0.0073511543785546</v>
       </c>
       <c r="AM132" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN132">
         <v>0.0171480510071521</v>
@@ -38076,7 +38079,7 @@
         <v>7436893.530962305</v>
       </c>
       <c r="CS132" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="CT132">
         <v>-0.8091587172086132</v>
@@ -38174,7 +38177,7 @@
         <v>0.0033730418087468</v>
       </c>
       <c r="AM133" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN133">
         <v>0.009616489085314</v>
@@ -38345,7 +38348,7 @@
         <v>867003.1587181734</v>
       </c>
       <c r="CS133" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="CT133">
         <v>-0.9000180936758766</v>
@@ -38443,7 +38446,7 @@
         <v>0.0074087938346481</v>
       </c>
       <c r="AM134" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN134">
         <v>0.0409391807131387</v>
@@ -38614,7 +38617,7 @@
         <v>3390202.150984915</v>
       </c>
       <c r="CS134" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="CT134">
         <v>-0.6893066803315582</v>
@@ -38712,7 +38715,7 @@
         <v>0.0083849241650579</v>
       </c>
       <c r="AM135" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN135">
         <v>0.0422126511911422</v>
@@ -38883,7 +38886,7 @@
         <v>8715912.703511165</v>
       </c>
       <c r="CS135" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="CT135">
         <v>-0.8034449984146571</v>
@@ -38981,7 +38984,7 @@
         <v>0.008401051909799701</v>
       </c>
       <c r="AM136" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN136">
         <v>0.020710590359547</v>
@@ -39152,7 +39155,7 @@
         <v>15549669.36335931</v>
       </c>
       <c r="CS136" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="CT136">
         <v>-0.8182238609422743</v>
@@ -39250,7 +39253,7 @@
         <v>0.0077330551594838</v>
       </c>
       <c r="AM137" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN137">
         <v>0.0190728510027463</v>
@@ -39421,7 +39424,7 @@
         <v>8185952.559251163</v>
       </c>
       <c r="CS137" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="CT137">
         <v>-0.8729982178980289</v>
@@ -39519,7 +39522,7 @@
         <v>0.010898810531027</v>
       </c>
       <c r="AM138" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN138">
         <v>0.035028448432581</v>
@@ -39690,7 +39693,7 @@
         <v>1792741.222718281</v>
       </c>
       <c r="CS138" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="CT138">
         <v>-0.7176955593761354</v>
@@ -39788,7 +39791,7 @@
         <v>0.0049947080562063</v>
       </c>
       <c r="AM139" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN139">
         <v>0.0090224491293264</v>
@@ -39959,7 +39962,7 @@
         <v>4157882.239708048</v>
       </c>
       <c r="CS139" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="CT139">
         <v>-0.8723102032515645</v>
@@ -40057,7 +40060,7 @@
         <v>0.006652001977027</v>
       </c>
       <c r="AM140" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN140">
         <v>0.0486790527459496</v>
@@ -40228,7 +40231,7 @@
         <v>7172478.294001529</v>
       </c>
       <c r="CS140" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="CT140">
         <v>-0.5365809810110987</v>
@@ -40326,7 +40329,7 @@
         <v>0.009892196288343501</v>
       </c>
       <c r="AM141" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN141">
         <v>0.0262045792935156</v>
@@ -40497,7 +40500,7 @@
         <v>10598803.27492217</v>
       </c>
       <c r="CS141" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="CT141">
         <v>-0.8043091815774359</v>
@@ -40595,7 +40598,7 @@
         <v>0.0032840087191214</v>
       </c>
       <c r="AM142" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN142">
         <v>0.011024599092909</v>
@@ -40766,7 +40769,7 @@
         <v>1954441.87495541</v>
       </c>
       <c r="CS142" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="CT142">
         <v>-0.892071333585829</v>
@@ -40864,7 +40867,7 @@
         <v>0.0042924384175561</v>
       </c>
       <c r="AM143" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN143">
         <v>0.0289399933126468</v>
@@ -41035,7 +41038,7 @@
         <v>2325567.261086872</v>
       </c>
       <c r="CS143" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="CT143">
         <v>-0.7586823863673019</v>
@@ -41133,7 +41136,7 @@
         <v>0.0066499576490462</v>
       </c>
       <c r="AM144" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN144">
         <v>0.0173750820094196</v>
@@ -41304,7 +41307,7 @@
         <v>17826610.98082536</v>
       </c>
       <c r="CS144" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="CT144">
         <v>-0.9111405881388872</v>
@@ -41402,7 +41405,7 @@
         <v>0.0095523432691301</v>
       </c>
       <c r="AM145" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN145">
         <v>0.0220904013262179</v>
@@ -41573,7 +41576,7 @@
         <v>2190979.247087742</v>
       </c>
       <c r="CS145" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="CT145">
         <v>-0.6948709396994353</v>
@@ -41671,7 +41674,7 @@
         <v>0.0112725621549946</v>
       </c>
       <c r="AM146" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN146">
         <v>0.0629290509487791</v>
@@ -41940,7 +41943,7 @@
         <v>0.01075541834616141</v>
       </c>
       <c r="AM147" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AN147">
         <v>0.07466532002742356</v>
@@ -42118,6 +42121,275 @@
       </c>
       <c r="CU147">
         <v>-0.8707969045725891</v>
+      </c>
+    </row>
+    <row r="148" spans="10:99">
+      <c r="J148" t="s">
+        <v>243</v>
+      </c>
+      <c r="K148">
+        <v>0.0008654450215017651</v>
+      </c>
+      <c r="L148">
+        <v>0.0008654450215017651</v>
+      </c>
+      <c r="M148">
+        <v>0.001646773835179527</v>
+      </c>
+      <c r="N148">
+        <v>0.001646773835179527</v>
+      </c>
+      <c r="O148">
+        <v>0.000991580787808899</v>
+      </c>
+      <c r="P148">
+        <v>0.000991580787808899</v>
+      </c>
+      <c r="Q148">
+        <v>0.001622732092626267</v>
+      </c>
+      <c r="R148">
+        <v>0.001622732092626267</v>
+      </c>
+      <c r="S148">
+        <v>8.983329450274754</v>
+      </c>
+      <c r="T148">
+        <v>8.249315530475144</v>
+      </c>
+      <c r="U148">
+        <v>0.9968107850618261</v>
+      </c>
+      <c r="V148">
+        <v>0.7091371326613198</v>
+      </c>
+      <c r="W148">
+        <v>0.08667258536559605</v>
+      </c>
+      <c r="X148">
+        <v>0.09793083597655818</v>
+      </c>
+      <c r="Y148">
+        <v>0.1890133841354915</v>
+      </c>
+      <c r="Z148">
+        <v>0.1721872846152441</v>
+      </c>
+      <c r="AA148">
+        <v>0.9985647018895669</v>
+      </c>
+      <c r="AB148">
+        <v>0.8351064625512248</v>
+      </c>
+      <c r="AC148">
+        <v>0.8646336939548427</v>
+      </c>
+      <c r="AD148">
+        <v>0.9967725907021084</v>
+      </c>
+      <c r="AE148">
+        <v>0.7992347746600847</v>
+      </c>
+      <c r="AF148">
+        <v>0.8298217557593828</v>
+      </c>
+      <c r="AG148">
+        <v>0.008743105624871524</v>
+      </c>
+      <c r="AH148">
+        <v>0.01216711024741432</v>
+      </c>
+      <c r="AI148">
+        <v>0.9985647018895669</v>
+      </c>
+      <c r="AJ148">
+        <v>0.9967725907021084</v>
+      </c>
+      <c r="AK148">
+        <v>0.008743105624871524</v>
+      </c>
+      <c r="AL148">
+        <v>0.01216711024741432</v>
+      </c>
+      <c r="AM148" t="s">
+        <v>244</v>
+      </c>
+      <c r="AN148">
+        <v>0.05947531493518945</v>
+      </c>
+      <c r="AO148">
+        <v>0.1274247914799327</v>
+      </c>
+      <c r="AP148">
+        <v>-551.7531234728001</v>
+      </c>
+      <c r="AQ148">
+        <v>-1961.6248515388</v>
+      </c>
+      <c r="AR148">
+        <v>25431.6692905271</v>
+      </c>
+      <c r="AS148">
+        <v>59026.72629646108</v>
+      </c>
+      <c r="AT148">
+        <v>25422.5117785271</v>
+      </c>
+      <c r="AU148">
+        <v>59026.72629646108</v>
+      </c>
+      <c r="AV148">
+        <v>1.543166929052711</v>
+      </c>
+      <c r="AW148">
+        <v>4.902672629646108</v>
+      </c>
+      <c r="AX148">
+        <v>2.671505709175953</v>
+      </c>
+      <c r="AY148">
+        <v>2.90958052434457</v>
+      </c>
+      <c r="AZ148">
+        <v>34.4</v>
+      </c>
+      <c r="BA148">
+        <v>38.53333333333333</v>
+      </c>
+      <c r="BB148">
+        <v>0.1031095913503279</v>
+      </c>
+      <c r="BC148">
+        <v>0.099712223438205</v>
+      </c>
+      <c r="BD148">
+        <v>-1837.508950473058</v>
+      </c>
+      <c r="BE148">
+        <v>-5647.263013868165</v>
+      </c>
+      <c r="BF148">
+        <v>2956</v>
+      </c>
+      <c r="BG148">
+        <v>4781</v>
+      </c>
+      <c r="BH148">
+        <v>1078.998611111111</v>
+      </c>
+      <c r="BI148">
+        <v>6737</v>
+      </c>
+      <c r="BJ148">
+        <v>4120</v>
+      </c>
+      <c r="BK148">
+        <v>9693</v>
+      </c>
+      <c r="BL148">
+        <v>8901</v>
+      </c>
+      <c r="BM148">
+        <v>0</v>
+      </c>
+      <c r="BN148">
+        <v>0</v>
+      </c>
+      <c r="BO148">
+        <v>128</v>
+      </c>
+      <c r="BP148">
+        <v>755</v>
+      </c>
+      <c r="BQ148">
+        <v>0</v>
+      </c>
+      <c r="BR148">
+        <v>0</v>
+      </c>
+      <c r="BS148">
+        <v>2828</v>
+      </c>
+      <c r="BT148">
+        <v>4026</v>
+      </c>
+      <c r="BU148">
+        <v>6737</v>
+      </c>
+      <c r="BV148">
+        <v>4120</v>
+      </c>
+      <c r="BW148">
+        <v>15431.66929052719</v>
+      </c>
+      <c r="BX148">
+        <v>49026.72629646119</v>
+      </c>
+      <c r="BY148">
+        <v>0.08907029222474379</v>
+      </c>
+      <c r="BZ148">
+        <v>0.08411163445231325</v>
+      </c>
+      <c r="CA148">
+        <v>0.2978207476223507</v>
+      </c>
+      <c r="CB148">
+        <v>0.1454284746387412</v>
+      </c>
+      <c r="CC148">
+        <v>0.01092990615565577</v>
+      </c>
+      <c r="CD148">
+        <v>0.01228844639671559</v>
+      </c>
+      <c r="CE148">
+        <v>0.0124999169776432</v>
+      </c>
+      <c r="CF148">
+        <v>0.01357124514220625</v>
+      </c>
+      <c r="CG148">
+        <v>15983.42241399999</v>
+      </c>
+      <c r="CH148">
+        <v>50988.35114799999</v>
+      </c>
+      <c r="CI148">
+        <v>17820.93136447304</v>
+      </c>
+      <c r="CJ148">
+        <v>56635.61416186816</v>
+      </c>
+      <c r="CK148">
+        <v>0.0897616575121067</v>
+      </c>
+      <c r="CL148">
+        <v>0.1179391706666686</v>
+      </c>
+      <c r="CM148">
+        <v>10000</v>
+      </c>
+      <c r="CO148">
+        <v>0.01463489979534309</v>
+      </c>
+      <c r="CP148">
+        <v>0.05116422751670078</v>
+      </c>
+      <c r="CQ148">
+        <v>22617300.28614038</v>
+      </c>
+      <c r="CR148">
+        <v>33517948.77339607</v>
+      </c>
+      <c r="CS148" s="2">
+        <v>45510.50511107766</v>
+      </c>
+      <c r="CT148">
+        <v>-0.7516800885976392</v>
+      </c>
+      <c r="CU148">
+        <v>-0.552387130925049</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update KAVAUSDT.json at 2024-08-06_20-20-07 bestfile_scores 0.00038195370088784926 bestfile_sharp 0.04076236855169546
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1129" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="388">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1539,7 +1539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU148"/>
+  <dimension ref="A1:CU149"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -42390,6 +42390,275 @@
       </c>
       <c r="CU148">
         <v>-0.552387130925049</v>
+      </c>
+    </row>
+    <row r="149" spans="10:99">
+      <c r="J149" t="s">
+        <v>239</v>
+      </c>
+      <c r="K149">
+        <v>0.001539670459458575</v>
+      </c>
+      <c r="L149">
+        <v>0.001539670459458575</v>
+      </c>
+      <c r="M149">
+        <v>0.000967767001506914</v>
+      </c>
+      <c r="N149">
+        <v>0.000967767001506914</v>
+      </c>
+      <c r="O149">
+        <v>0.001528178840837024</v>
+      </c>
+      <c r="P149">
+        <v>0.001528178840837024</v>
+      </c>
+      <c r="Q149">
+        <v>0.0008568539482927795</v>
+      </c>
+      <c r="R149">
+        <v>0.0008568539482927795</v>
+      </c>
+      <c r="S149">
+        <v>25.55543558417511</v>
+      </c>
+      <c r="T149">
+        <v>10.43389564174606</v>
+      </c>
+      <c r="U149">
+        <v>0.9903830827773132</v>
+      </c>
+      <c r="V149">
+        <v>0.6983167081863534</v>
+      </c>
+      <c r="W149">
+        <v>0.07767822502634231</v>
+      </c>
+      <c r="X149">
+        <v>0.07619329814793283</v>
+      </c>
+      <c r="Y149">
+        <v>0.2265564135738889</v>
+      </c>
+      <c r="Z149">
+        <v>0.177853027024439</v>
+      </c>
+      <c r="AA149">
+        <v>0.9983501622472053</v>
+      </c>
+      <c r="AB149">
+        <v>0.8566234782846035</v>
+      </c>
+      <c r="AC149">
+        <v>0.8380233689002388</v>
+      </c>
+      <c r="AD149">
+        <v>0.9982271555000344</v>
+      </c>
+      <c r="AE149">
+        <v>0.7736909263770486</v>
+      </c>
+      <c r="AF149">
+        <v>0.8223674871415904</v>
+      </c>
+      <c r="AG149">
+        <v>0.00863693076930128</v>
+      </c>
+      <c r="AH149">
+        <v>0.008640155143380991</v>
+      </c>
+      <c r="AI149">
+        <v>0.9983501622472053</v>
+      </c>
+      <c r="AJ149">
+        <v>0.9982271555000344</v>
+      </c>
+      <c r="AK149">
+        <v>0.00863693076930128</v>
+      </c>
+      <c r="AL149">
+        <v>0.008640155143380991</v>
+      </c>
+      <c r="AM149" t="s">
+        <v>244</v>
+      </c>
+      <c r="AN149">
+        <v>0.07371412979936612</v>
+      </c>
+      <c r="AO149">
+        <v>0.05717297154639175</v>
+      </c>
+      <c r="AP149">
+        <v>-1856.69298268</v>
+      </c>
+      <c r="AQ149">
+        <v>-483.25193874</v>
+      </c>
+      <c r="AR149">
+        <v>40356.99241732022</v>
+      </c>
+      <c r="AS149">
+        <v>24041.51726126008</v>
+      </c>
+      <c r="AT149">
+        <v>40355.13961732022</v>
+      </c>
+      <c r="AU149">
+        <v>24038.10026126008</v>
+      </c>
+      <c r="AV149">
+        <v>3.035699241732022</v>
+      </c>
+      <c r="AW149">
+        <v>1.404151726126007</v>
+      </c>
+      <c r="AX149">
+        <v>0.9391509162567245</v>
+      </c>
+      <c r="AY149">
+        <v>2.300007046471479</v>
+      </c>
+      <c r="AZ149">
+        <v>37.93333333333333</v>
+      </c>
+      <c r="BA149">
+        <v>41.28333333333333</v>
+      </c>
+      <c r="BB149">
+        <v>0.07609453288998462</v>
+      </c>
+      <c r="BC149">
+        <v>0.07532181822408669</v>
+      </c>
+      <c r="BD149">
+        <v>-2653.177657715952</v>
+      </c>
+      <c r="BE149">
+        <v>-1183.148956027105</v>
+      </c>
+      <c r="BF149">
+        <v>7830</v>
+      </c>
+      <c r="BG149">
+        <v>5405</v>
+      </c>
+      <c r="BH149">
+        <v>906.8520833333333</v>
+      </c>
+      <c r="BI149">
+        <v>15345</v>
+      </c>
+      <c r="BJ149">
+        <v>4057</v>
+      </c>
+      <c r="BK149">
+        <v>23175</v>
+      </c>
+      <c r="BL149">
+        <v>9462</v>
+      </c>
+      <c r="BM149">
+        <v>0</v>
+      </c>
+      <c r="BN149">
+        <v>0</v>
+      </c>
+      <c r="BO149">
+        <v>3750</v>
+      </c>
+      <c r="BP149">
+        <v>732</v>
+      </c>
+      <c r="BQ149">
+        <v>0</v>
+      </c>
+      <c r="BR149">
+        <v>0</v>
+      </c>
+      <c r="BS149">
+        <v>4080</v>
+      </c>
+      <c r="BT149">
+        <v>4673</v>
+      </c>
+      <c r="BU149">
+        <v>15345</v>
+      </c>
+      <c r="BV149">
+        <v>4057</v>
+      </c>
+      <c r="BW149">
+        <v>30356.99241731995</v>
+      </c>
+      <c r="BX149">
+        <v>14041.51726126001</v>
+      </c>
+      <c r="BY149">
+        <v>0.07944929949855256</v>
+      </c>
+      <c r="BZ149">
+        <v>0.07290428891734235</v>
+      </c>
+      <c r="CA149">
+        <v>0.2939414045616529</v>
+      </c>
+      <c r="CB149">
+        <v>0.1508373732980492</v>
+      </c>
+      <c r="CC149">
+        <v>0.008541457371382059</v>
+      </c>
+      <c r="CD149">
+        <v>0.01502445815399398</v>
+      </c>
+      <c r="CE149">
+        <v>0.01132079572183098</v>
+      </c>
+      <c r="CF149">
+        <v>0.01358610203418608</v>
+      </c>
+      <c r="CG149">
+        <v>32213.68539999995</v>
+      </c>
+      <c r="CH149">
+        <v>14524.76920000001</v>
+      </c>
+      <c r="CI149">
+        <v>34866.8630577159</v>
+      </c>
+      <c r="CJ149">
+        <v>15707.91815602711</v>
+      </c>
+      <c r="CK149">
+        <v>0.1826593380074046</v>
+      </c>
+      <c r="CL149">
+        <v>0.09736031104338029</v>
+      </c>
+      <c r="CM149">
+        <v>10000</v>
+      </c>
+      <c r="CO149">
+        <v>0.03349260314251585</v>
+      </c>
+      <c r="CP149">
+        <v>0.01741247817697326</v>
+      </c>
+      <c r="CQ149">
+        <v>58107883.34426937</v>
+      </c>
+      <c r="CR149">
+        <v>9758740.845571002</v>
+      </c>
+      <c r="CS149" s="2">
+        <v>45510.63778221698</v>
+      </c>
+      <c r="CT149">
+        <v>-0.7358834399820444</v>
+      </c>
+      <c r="CU149">
+        <v>-0.7141006607483422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update LINKUSDT.json at 2024-08-07_00-44-46 bestfile_scores 0.0005493991930936082 bestfile_sharp 0.0997444423370649
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="387">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -743,9 +743,6 @@
   </si>
   <si>
     <t>HNTUSDT</t>
-  </si>
-  <si>
-    <t>HOTUSDT</t>
   </si>
   <si>
     <t>binance</t>
@@ -1539,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU149"/>
+  <dimension ref="A1:CU146"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1954,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN2">
         <v>0.049606857</v>
@@ -2119,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="CS2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:99">
@@ -2235,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="AM3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN3">
         <v>0.04006526</v>
@@ -2400,7 +2397,7 @@
         <v>0</v>
       </c>
       <c r="CS3" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:99">
@@ -2516,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN4">
         <v>0.092575794</v>
@@ -2681,7 +2678,7 @@
         <v>0</v>
       </c>
       <c r="CS4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:99">
@@ -2797,7 +2794,7 @@
         <v>0</v>
       </c>
       <c r="AM5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN5">
         <v>0.027448502</v>
@@ -2962,7 +2959,7 @@
         <v>0</v>
       </c>
       <c r="CS5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:99">
@@ -3078,7 +3075,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN6">
         <v>0.083929868</v>
@@ -3243,7 +3240,7 @@
         <v>0</v>
       </c>
       <c r="CS6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:99">
@@ -3359,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN7">
         <v>0.145376251</v>
@@ -3524,7 +3521,7 @@
         <v>0</v>
       </c>
       <c r="CS7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:99">
@@ -3640,7 +3637,7 @@
         <v>0</v>
       </c>
       <c r="AM8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN8">
         <v>0.087987204</v>
@@ -3805,7 +3802,7 @@
         <v>0</v>
       </c>
       <c r="CS8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:99">
@@ -3921,7 +3918,7 @@
         <v>0</v>
       </c>
       <c r="AM9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN9">
         <v>0.118237951</v>
@@ -4086,7 +4083,7 @@
         <v>0</v>
       </c>
       <c r="CS9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:99">
@@ -4202,7 +4199,7 @@
         <v>0</v>
       </c>
       <c r="AM10" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN10">
         <v>0.08106915200000001</v>
@@ -4367,7 +4364,7 @@
         <v>0</v>
       </c>
       <c r="CS10" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:99">
@@ -4483,7 +4480,7 @@
         <v>0</v>
       </c>
       <c r="AM11" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN11">
         <v>0.027960571</v>
@@ -4648,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="CS11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:99">
@@ -4764,7 +4761,7 @@
         <v>0</v>
       </c>
       <c r="AM12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN12">
         <v>0.032951036</v>
@@ -4929,7 +4926,7 @@
         <v>0</v>
       </c>
       <c r="CS12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:99">
@@ -5045,7 +5042,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN13">
         <v>0.179185242</v>
@@ -5210,7 +5207,7 @@
         <v>0</v>
       </c>
       <c r="CS13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:99">
@@ -5326,7 +5323,7 @@
         <v>0</v>
       </c>
       <c r="AM14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN14">
         <v>0.143233482</v>
@@ -5491,7 +5488,7 @@
         <v>0</v>
       </c>
       <c r="CS14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:99">
@@ -5607,7 +5604,7 @@
         <v>0</v>
       </c>
       <c r="AM15" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN15">
         <v>0.138115134</v>
@@ -5772,7 +5769,7 @@
         <v>0</v>
       </c>
       <c r="CS15" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:99">
@@ -5888,7 +5885,7 @@
         <v>0</v>
       </c>
       <c r="AM16" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN16">
         <v>0.09650975000000001</v>
@@ -6053,7 +6050,7 @@
         <v>0</v>
       </c>
       <c r="CS16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:97">
@@ -6169,7 +6166,7 @@
         <v>0</v>
       </c>
       <c r="AM17" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN17">
         <v>0.060693695</v>
@@ -6334,7 +6331,7 @@
         <v>0</v>
       </c>
       <c r="CS17" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:97">
@@ -6450,7 +6447,7 @@
         <v>0</v>
       </c>
       <c r="AM18" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN18">
         <v>0.107514363</v>
@@ -6615,7 +6612,7 @@
         <v>0</v>
       </c>
       <c r="CS18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:97">
@@ -6731,7 +6728,7 @@
         <v>0</v>
       </c>
       <c r="AM19" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN19">
         <v>0.014898256</v>
@@ -6896,7 +6893,7 @@
         <v>0</v>
       </c>
       <c r="CS19" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:97">
@@ -7012,7 +7009,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN20">
         <v>0.02858403</v>
@@ -7177,7 +7174,7 @@
         <v>0</v>
       </c>
       <c r="CS20" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:97">
@@ -7293,7 +7290,7 @@
         <v>0</v>
       </c>
       <c r="AM21" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN21">
         <v>0.082273481</v>
@@ -7458,7 +7455,7 @@
         <v>0</v>
       </c>
       <c r="CS21" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:97">
@@ -7574,7 +7571,7 @@
         <v>0</v>
       </c>
       <c r="AM22" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN22">
         <v>0.012592558</v>
@@ -7739,7 +7736,7 @@
         <v>0</v>
       </c>
       <c r="CS22" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:97">
@@ -7855,7 +7852,7 @@
         <v>0</v>
       </c>
       <c r="AM23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN23">
         <v>0.00903967</v>
@@ -8020,7 +8017,7 @@
         <v>0</v>
       </c>
       <c r="CS23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:97">
@@ -8136,7 +8133,7 @@
         <v>0</v>
       </c>
       <c r="AM24" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN24">
         <v>0.030046089</v>
@@ -8301,7 +8298,7 @@
         <v>0</v>
       </c>
       <c r="CS24" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:97">
@@ -8417,7 +8414,7 @@
         <v>0</v>
       </c>
       <c r="AM25" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN25">
         <v>0.010607012</v>
@@ -8582,7 +8579,7 @@
         <v>0</v>
       </c>
       <c r="CS25" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:97">
@@ -8698,7 +8695,7 @@
         <v>0</v>
       </c>
       <c r="AM26" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN26">
         <v>0.053096335</v>
@@ -8863,7 +8860,7 @@
         <v>0</v>
       </c>
       <c r="CS26" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="27" spans="1:97">
@@ -8979,7 +8976,7 @@
         <v>0</v>
       </c>
       <c r="AM27" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN27">
         <v>0.092674047</v>
@@ -9144,7 +9141,7 @@
         <v>0</v>
       </c>
       <c r="CS27" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:97">
@@ -9260,7 +9257,7 @@
         <v>0</v>
       </c>
       <c r="AM28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN28">
         <v>0.03099706</v>
@@ -9425,7 +9422,7 @@
         <v>0</v>
       </c>
       <c r="CS28" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:97">
@@ -9541,7 +9538,7 @@
         <v>0</v>
       </c>
       <c r="AM29" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN29">
         <v>0.069423731</v>
@@ -9706,7 +9703,7 @@
         <v>0</v>
       </c>
       <c r="CS29" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:97">
@@ -9822,7 +9819,7 @@
         <v>0</v>
       </c>
       <c r="AM30" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN30">
         <v>0.060424834</v>
@@ -9987,7 +9984,7 @@
         <v>0</v>
       </c>
       <c r="CS30" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:97">
@@ -10103,7 +10100,7 @@
         <v>0</v>
       </c>
       <c r="AM31" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN31">
         <v>0.056666776</v>
@@ -10268,7 +10265,7 @@
         <v>0</v>
       </c>
       <c r="CS31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:97">
@@ -10384,7 +10381,7 @@
         <v>0</v>
       </c>
       <c r="AM32" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN32">
         <v>0.098888062</v>
@@ -10549,7 +10546,7 @@
         <v>0</v>
       </c>
       <c r="CS32" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:99">
@@ -10665,7 +10662,7 @@
         <v>0</v>
       </c>
       <c r="AM33" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN33">
         <v>0.035815903</v>
@@ -10830,7 +10827,7 @@
         <v>0</v>
       </c>
       <c r="CS33" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="34" spans="1:99">
@@ -10946,7 +10943,7 @@
         <v>0</v>
       </c>
       <c r="AM34" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN34">
         <v>0.037311133</v>
@@ -11111,7 +11108,7 @@
         <v>0</v>
       </c>
       <c r="CS34" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="CT34">
         <v>-0.814742818</v>
@@ -11233,7 +11230,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN35">
         <v>0.041330496</v>
@@ -11398,7 +11395,7 @@
         <v>0</v>
       </c>
       <c r="CS35" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="CT35">
         <v>-0.753066891</v>
@@ -11520,7 +11517,7 @@
         <v>0</v>
       </c>
       <c r="AM36" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN36">
         <v>0.047772102</v>
@@ -11685,7 +11682,7 @@
         <v>0</v>
       </c>
       <c r="CS36" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="CT36">
         <v>-0.872335259</v>
@@ -11807,7 +11804,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN37">
         <v>0.060484521</v>
@@ -11972,7 +11969,7 @@
         <v>0</v>
       </c>
       <c r="CS37" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="CT37">
         <v>-0.759885442</v>
@@ -12094,7 +12091,7 @@
         <v>0</v>
       </c>
       <c r="AM38" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN38">
         <v>0.061007062</v>
@@ -12259,7 +12256,7 @@
         <v>0</v>
       </c>
       <c r="CS38" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="CT38">
         <v>-0.838900609</v>
@@ -12381,7 +12378,7 @@
         <v>0</v>
       </c>
       <c r="AM39" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN39">
         <v>0.025236369</v>
@@ -12546,7 +12543,7 @@
         <v>0</v>
       </c>
       <c r="CS39" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="CT39">
         <v>-0.780218664</v>
@@ -12668,7 +12665,7 @@
         <v>0</v>
       </c>
       <c r="AM40" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN40">
         <v>0.031804424</v>
@@ -12833,7 +12830,7 @@
         <v>0</v>
       </c>
       <c r="CS40" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="CT40">
         <v>-0.79992089</v>
@@ -12955,7 +12952,7 @@
         <v>0</v>
       </c>
       <c r="AM41" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN41">
         <v>0.072404657</v>
@@ -13120,7 +13117,7 @@
         <v>0</v>
       </c>
       <c r="CS41" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="CT41">
         <v>-0.528089775</v>
@@ -13242,7 +13239,7 @@
         <v>0</v>
       </c>
       <c r="AM42" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN42">
         <v>0.06821192299999999</v>
@@ -13407,7 +13404,7 @@
         <v>0</v>
       </c>
       <c r="CS42" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="CT42">
         <v>-0.754849911</v>
@@ -13529,7 +13526,7 @@
         <v>0</v>
       </c>
       <c r="AM43" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN43">
         <v>0.069326524</v>
@@ -13694,7 +13691,7 @@
         <v>0</v>
       </c>
       <c r="CS43" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="CT43">
         <v>-0.7655395739999999</v>
@@ -13816,7 +13813,7 @@
         <v>0</v>
       </c>
       <c r="AM44" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN44">
         <v>0.036991009</v>
@@ -13981,7 +13978,7 @@
         <v>0</v>
       </c>
       <c r="CS44" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="CT44">
         <v>-0.829764531</v>
@@ -14103,7 +14100,7 @@
         <v>0</v>
       </c>
       <c r="AM45" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN45">
         <v>0.036729519</v>
@@ -14268,7 +14265,7 @@
         <v>0</v>
       </c>
       <c r="CS45" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="CT45">
         <v>-0.404237806</v>
@@ -14390,7 +14387,7 @@
         <v>0</v>
       </c>
       <c r="AM46" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN46">
         <v>0.045071814</v>
@@ -14555,7 +14552,7 @@
         <v>0</v>
       </c>
       <c r="CS46" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="CT46">
         <v>-0.703677808</v>
@@ -14677,7 +14674,7 @@
         <v>0</v>
       </c>
       <c r="AM47" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN47">
         <v>0.0580535</v>
@@ -14842,7 +14839,7 @@
         <v>0</v>
       </c>
       <c r="CS47" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="CT47">
         <v>-0.753715321</v>
@@ -14964,7 +14961,7 @@
         <v>0</v>
       </c>
       <c r="AM48" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN48">
         <v>0.056639031</v>
@@ -15129,7 +15126,7 @@
         <v>0</v>
       </c>
       <c r="CS48" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="CT48">
         <v>-0.71793867</v>
@@ -15251,7 +15248,7 @@
         <v>0</v>
       </c>
       <c r="AM49" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN49">
         <v>0.074241638</v>
@@ -15416,7 +15413,7 @@
         <v>0</v>
       </c>
       <c r="CS49" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="CT49">
         <v>-0.655169358</v>
@@ -15538,7 +15535,7 @@
         <v>0</v>
       </c>
       <c r="AM50" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN50">
         <v>0.05430774</v>
@@ -15703,7 +15700,7 @@
         <v>0</v>
       </c>
       <c r="CS50" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="CT50">
         <v>-0.6872439380000001</v>
@@ -15825,7 +15822,7 @@
         <v>0</v>
       </c>
       <c r="AM51" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN51">
         <v>0.080539377</v>
@@ -15990,7 +15987,7 @@
         <v>0</v>
       </c>
       <c r="CS51" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="CT51">
         <v>-0.596275172</v>
@@ -16112,7 +16109,7 @@
         <v>0</v>
       </c>
       <c r="AM52" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN52">
         <v>0.032588051</v>
@@ -16277,7 +16274,7 @@
         <v>0</v>
       </c>
       <c r="CS52" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="CT52">
         <v>-0.808081961</v>
@@ -16399,7 +16396,7 @@
         <v>0</v>
       </c>
       <c r="AM53" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN53">
         <v>0.026475554</v>
@@ -16564,7 +16561,7 @@
         <v>0</v>
       </c>
       <c r="CS53" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="CT53">
         <v>-0.77227813</v>
@@ -16686,7 +16683,7 @@
         <v>0</v>
       </c>
       <c r="AM54" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN54">
         <v>0.0245106310926154</v>
@@ -16851,7 +16848,7 @@
         <v>0</v>
       </c>
       <c r="CS54" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="CT54">
         <v>-0.8664117478627688</v>
@@ -16970,7 +16967,7 @@
         <v>0</v>
       </c>
       <c r="AM55" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN55">
         <v>0.0779439577559576</v>
@@ -17135,7 +17132,7 @@
         <v>0</v>
       </c>
       <c r="CS55" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="CT55">
         <v>-0.7108907987632488</v>
@@ -17251,7 +17248,7 @@
         <v>0</v>
       </c>
       <c r="AM56" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN56">
         <v>0.0402740604837066</v>
@@ -17416,7 +17413,7 @@
         <v>0</v>
       </c>
       <c r="CS56" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="CT56">
         <v>-0.7447372903525753</v>
@@ -17529,7 +17526,7 @@
         <v>0</v>
       </c>
       <c r="AM57" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN57">
         <v>0.0441363962743036</v>
@@ -17694,7 +17691,7 @@
         <v>0</v>
       </c>
       <c r="CS57" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="CT57">
         <v>-0.7777179486581601</v>
@@ -17807,7 +17804,7 @@
         <v>0</v>
       </c>
       <c r="AM58" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN58">
         <v>0.0589646348207879</v>
@@ -17972,7 +17969,7 @@
         <v>0</v>
       </c>
       <c r="CS58" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="CT58">
         <v>-0.7757098341832183</v>
@@ -18085,7 +18082,7 @@
         <v>0</v>
       </c>
       <c r="AM59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN59">
         <v>0.0088498418945465</v>
@@ -18250,7 +18247,7 @@
         <v>0</v>
       </c>
       <c r="CS59" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="CT59">
         <v>-0.9614802262041642</v>
@@ -18363,7 +18360,7 @@
         <v>0</v>
       </c>
       <c r="AM60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN60">
         <v>0.0438527807624406</v>
@@ -18528,7 +18525,7 @@
         <v>0</v>
       </c>
       <c r="CS60" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="CT60">
         <v>-0.6569921650581255</v>
@@ -18641,7 +18638,7 @@
         <v>0</v>
       </c>
       <c r="AM61" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN61">
         <v>0.0175722673111926</v>
@@ -18806,7 +18803,7 @@
         <v>0</v>
       </c>
       <c r="CS61" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="CT61">
         <v>-0.924044412704054</v>
@@ -18919,7 +18916,7 @@
         <v>0</v>
       </c>
       <c r="AM62" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN62">
         <v>0.0551224625318549</v>
@@ -19084,7 +19081,7 @@
         <v>0</v>
       </c>
       <c r="CS62" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="CT62">
         <v>-0.6213262971882773</v>
@@ -19197,7 +19194,7 @@
         <v>0</v>
       </c>
       <c r="AM63" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN63">
         <v>0.0157574961492794</v>
@@ -19362,7 +19359,7 @@
         <v>0</v>
       </c>
       <c r="CS63" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="CT63">
         <v>-0.9477002142299265</v>
@@ -19475,7 +19472,7 @@
         <v>0</v>
       </c>
       <c r="AM64" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN64">
         <v>0.0348775184726272</v>
@@ -19640,7 +19637,7 @@
         <v>0</v>
       </c>
       <c r="CS64" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="CT64">
         <v>-0.7774025388699596</v>
@@ -19753,7 +19750,7 @@
         <v>0</v>
       </c>
       <c r="AM65" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN65">
         <v>0.0617007650932976</v>
@@ -19918,7 +19915,7 @@
         <v>0</v>
       </c>
       <c r="CS65" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="CT65">
         <v>-0.8140402180385446</v>
@@ -20031,7 +20028,7 @@
         <v>0.0108330657640134</v>
       </c>
       <c r="AM66" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN66">
         <v>0.0122896465671382</v>
@@ -20202,7 +20199,7 @@
         <v>28802806.1197283</v>
       </c>
       <c r="CS66" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="CT66">
         <v>-0.7661604887809055</v>
@@ -20315,7 +20312,7 @@
         <v>0.009662114019183699</v>
       </c>
       <c r="AM67" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN67">
         <v>0.0157075521173083</v>
@@ -20486,7 +20483,7 @@
         <v>12816652.38654842</v>
       </c>
       <c r="CS67" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="CT67">
         <v>-0.843107865610227</v>
@@ -20599,7 +20596,7 @@
         <v>0.009682496602030599</v>
       </c>
       <c r="AM68" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN68">
         <v>0.019453807476403</v>
@@ -20770,7 +20767,7 @@
         <v>362119.31393403</v>
       </c>
       <c r="CS68" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="CT68">
         <v>-0.7040504011377985</v>
@@ -20883,7 +20880,7 @@
         <v>0.009502809785555901</v>
       </c>
       <c r="AM69" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN69">
         <v>0.0467996269477206</v>
@@ -21054,7 +21051,7 @@
         <v>3444392.687119505</v>
       </c>
       <c r="CS69" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="CT69">
         <v>-0.5814104972412503</v>
@@ -21164,7 +21161,7 @@
         <v>0.0100375716524098</v>
       </c>
       <c r="AM70" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN70">
         <v>0.0260012684361012</v>
@@ -21335,7 +21332,7 @@
         <v>8020410.490554446</v>
       </c>
       <c r="CS70" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="CT70">
         <v>-0.1225754953154068</v>
@@ -21442,7 +21439,7 @@
         <v>0.0030270679524292</v>
       </c>
       <c r="AM71" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN71">
         <v>0.007629803458883</v>
@@ -21613,7 +21610,7 @@
         <v>6690404.196816532</v>
       </c>
       <c r="CS71" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="CT71">
         <v>-0.943556327266077</v>
@@ -21717,7 +21714,7 @@
         <v>0.0071318120684325</v>
       </c>
       <c r="AM72" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN72">
         <v>0.0106438024257861</v>
@@ -21888,7 +21885,7 @@
         <v>2333580.086114224</v>
       </c>
       <c r="CS72" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="CT72">
         <v>-0.9017649135974464</v>
@@ -21992,7 +21989,7 @@
         <v>0.008671749707596699</v>
       </c>
       <c r="AM73" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN73">
         <v>0.008922434565822699</v>
@@ -22163,7 +22160,7 @@
         <v>4050354.030474017</v>
       </c>
       <c r="CS73" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="CT73">
         <v>-0.9011542748767548</v>
@@ -22267,7 +22264,7 @@
         <v>0.0061287699408089</v>
       </c>
       <c r="AM74" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN74">
         <v>0.0100444206462455</v>
@@ -22438,7 +22435,7 @@
         <v>284228.7150822567</v>
       </c>
       <c r="CS74" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="CT74">
         <v>-0.9022640234515124</v>
@@ -22542,7 +22539,7 @@
         <v>0.009112086818146899</v>
       </c>
       <c r="AM75" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN75">
         <v>0.0105885988628848</v>
@@ -22713,7 +22710,7 @@
         <v>9238253.926865038</v>
       </c>
       <c r="CS75" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="CT75">
         <v>-0.8442464713130005</v>
@@ -22817,7 +22814,7 @@
         <v>0.0120332146147572</v>
       </c>
       <c r="AM76" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN76">
         <v>0.005689041712621</v>
@@ -22988,7 +22985,7 @@
         <v>103761437.1558867</v>
       </c>
       <c r="CS76" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="CT76">
         <v>-0.9172425776350784</v>
@@ -23092,7 +23089,7 @@
         <v>0.009980777925547499</v>
       </c>
       <c r="AM77" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN77">
         <v>0.0213191472253163</v>
@@ -23263,7 +23260,7 @@
         <v>11075597.03060125</v>
       </c>
       <c r="CS77" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="CT77">
         <v>-0.7048134977852135</v>
@@ -23364,7 +23361,7 @@
         <v>0.008640349693688199</v>
       </c>
       <c r="AM78" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN78">
         <v>0.0310379691662141</v>
@@ -23535,7 +23532,7 @@
         <v>4941591.885046311</v>
       </c>
       <c r="CS78" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="CT78">
         <v>-0.6921566954508142</v>
@@ -23636,7 +23633,7 @@
         <v>0.0052151469726826</v>
       </c>
       <c r="AM79" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN79">
         <v>0.0187749711217366</v>
@@ -23807,7 +23804,7 @@
         <v>13794144.77050867</v>
       </c>
       <c r="CS79" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="CT79">
         <v>-0.6546270123512354</v>
@@ -23908,7 +23905,7 @@
         <v>0.0083235819058295</v>
       </c>
       <c r="AM80" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN80">
         <v>0.0531066176371749</v>
@@ -24079,7 +24076,7 @@
         <v>1271425.087705649</v>
       </c>
       <c r="CS80" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="CT80">
         <v>-0.3384511866527668</v>
@@ -24180,7 +24177,7 @@
         <v>0.0041067346844988</v>
       </c>
       <c r="AM81" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN81">
         <v>0.0376358519870464</v>
@@ -24351,7 +24348,7 @@
         <v>8472790.733285822</v>
       </c>
       <c r="CS81" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="CT81">
         <v>-0.5869016106017596</v>
@@ -24452,7 +24449,7 @@
         <v>0.0055266741344329</v>
       </c>
       <c r="AM82" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN82">
         <v>0.0047447694558675</v>
@@ -24623,7 +24620,7 @@
         <v>6299784.652790904</v>
       </c>
       <c r="CS82" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="CT82">
         <v>-0.9571664073286058</v>
@@ -24724,7 +24721,7 @@
         <v>0.0083610158619657</v>
       </c>
       <c r="AM83" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN83">
         <v>0.0075895877096284</v>
@@ -24895,7 +24892,7 @@
         <v>9553962.229671104</v>
       </c>
       <c r="CS83" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="CT83">
         <v>-0.7975627900619038</v>
@@ -24996,7 +24993,7 @@
         <v>0.0110102665992773</v>
       </c>
       <c r="AM84" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN84">
         <v>0.0289129415567337</v>
@@ -25167,7 +25164,7 @@
         <v>9017755.465507764</v>
       </c>
       <c r="CS84" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="CT84">
         <v>-0.641321453686593</v>
@@ -25265,7 +25262,7 @@
         <v>0.001235474151197</v>
       </c>
       <c r="AM85" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN85">
         <v>0.0236860634403801</v>
@@ -25436,7 +25433,7 @@
         <v>395804.1998002621</v>
       </c>
       <c r="CS85" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="CT85">
         <v>-0.8468525619890503</v>
@@ -25534,7 +25531,7 @@
         <v>0.0069339646256509</v>
       </c>
       <c r="AM86" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN86">
         <v>0.0046798420774097</v>
@@ -25705,7 +25702,7 @@
         <v>5470308.140646266</v>
       </c>
       <c r="CS86" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="CT86">
         <v>-0.9414869172232342</v>
@@ -25803,7 +25800,7 @@
         <v>0.0084303895709902</v>
       </c>
       <c r="AM87" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN87">
         <v>0.0220548762227611</v>
@@ -25974,7 +25971,7 @@
         <v>10570112.91971009</v>
       </c>
       <c r="CS87" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="CT87">
         <v>-0.8207903291654746</v>
@@ -26072,7 +26069,7 @@
         <v>0.0046858616922062</v>
       </c>
       <c r="AM88" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN88">
         <v>0.0514935425696241</v>
@@ -26243,7 +26240,7 @@
         <v>5725644.496349121</v>
       </c>
       <c r="CS88" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="CT88">
         <v>-0.561712415905279</v>
@@ -26341,7 +26338,7 @@
         <v>0.0039939215766598</v>
       </c>
       <c r="AM89" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN89">
         <v>0.012222058764571</v>
@@ -26512,7 +26509,7 @@
         <v>1429804.32644608</v>
       </c>
       <c r="CS89" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="CT89">
         <v>-0.9176379634509604</v>
@@ -26610,7 +26607,7 @@
         <v>0.0042088758977745</v>
       </c>
       <c r="AM90" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN90">
         <v>0.019939030911244</v>
@@ -26781,7 +26778,7 @@
         <v>4722406.067514317</v>
       </c>
       <c r="CS90" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="CT90">
         <v>-0.9278452363120948</v>
@@ -26879,7 +26876,7 @@
         <v>0.0090603002679094</v>
       </c>
       <c r="AM91" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN91">
         <v>0.0130335524359802</v>
@@ -27050,7 +27047,7 @@
         <v>2899232.912138085</v>
       </c>
       <c r="CS91" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="CT91">
         <v>-0.8179686291978085</v>
@@ -27148,7 +27145,7 @@
         <v>0.0034278853232647</v>
       </c>
       <c r="AM92" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN92">
         <v>0.0267226315229668</v>
@@ -27319,7 +27316,7 @@
         <v>1448171.53934798</v>
       </c>
       <c r="CS92" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="CT92">
         <v>-0.8215150584575165</v>
@@ -27417,7 +27414,7 @@
         <v>0.0078801601208179</v>
       </c>
       <c r="AM93" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN93">
         <v>0.0221393128933173</v>
@@ -27588,7 +27585,7 @@
         <v>16635452.15900955</v>
       </c>
       <c r="CS93" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="CT93">
         <v>-0.7542388832888753</v>
@@ -27686,7 +27683,7 @@
         <v>0.0148358454007108</v>
       </c>
       <c r="AM94" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN94">
         <v>0.0142895129437342</v>
@@ -27857,7 +27854,7 @@
         <v>118847.66881</v>
       </c>
       <c r="CS94" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="CT94">
         <v>-0.8706219162560768</v>
@@ -27955,7 +27952,7 @@
         <v>0.00777307269066</v>
       </c>
       <c r="AM95" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN95">
         <v>0.028345432375321</v>
@@ -28126,7 +28123,7 @@
         <v>9989976.067409206</v>
       </c>
       <c r="CS95" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="CT95">
         <v>-0.7702665229627835</v>
@@ -28224,7 +28221,7 @@
         <v>0.005069566938105</v>
       </c>
       <c r="AM96" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN96">
         <v>0.0378882038525435</v>
@@ -28395,7 +28392,7 @@
         <v>4195010.116009732</v>
       </c>
       <c r="CS96" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="CT96">
         <v>-0.6208027078099908</v>
@@ -28493,7 +28490,7 @@
         <v>0.0109181034800677</v>
       </c>
       <c r="AM97" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN97">
         <v>0.0464479162381462</v>
@@ -28664,7 +28661,7 @@
         <v>1753546.300271091</v>
       </c>
       <c r="CS97" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="CT97">
         <v>-0.6637406607330143</v>
@@ -28762,7 +28759,7 @@
         <v>0.0073561352130028</v>
       </c>
       <c r="AM98" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN98">
         <v>0.0129973328606765</v>
@@ -28933,7 +28930,7 @@
         <v>8525723.260530123</v>
       </c>
       <c r="CS98" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="CT98">
         <v>-0.6066396906320848</v>
@@ -29031,7 +29028,7 @@
         <v>0.0010483764611907</v>
       </c>
       <c r="AM99" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN99">
         <v>0.0224095392580651</v>
@@ -29202,7 +29199,7 @@
         <v>555000.5818001842</v>
       </c>
       <c r="CS99" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="CT99">
         <v>-0.7930559623825889</v>
@@ -29300,7 +29297,7 @@
         <v>0.0034227206580065</v>
       </c>
       <c r="AM100" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN100">
         <v>0.0120356538583077</v>
@@ -29471,7 +29468,7 @@
         <v>8829982.660321526</v>
       </c>
       <c r="CS100" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="CT100">
         <v>-0.8625963918106255</v>
@@ -29569,7 +29566,7 @@
         <v>0.0024512168149686</v>
       </c>
       <c r="AM101" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN101">
         <v>0.0237148028402029</v>
@@ -29740,7 +29737,7 @@
         <v>3109464.939265249</v>
       </c>
       <c r="CS101" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="CT101">
         <v>-0.8320151516141147</v>
@@ -29838,7 +29835,7 @@
         <v>0.0013136523187938</v>
       </c>
       <c r="AM102" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN102">
         <v>0.0039597254802618</v>
@@ -30009,7 +30006,7 @@
         <v>1199182.410839436</v>
       </c>
       <c r="CS102" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="CT102">
         <v>-0.9034091343725908</v>
@@ -30107,7 +30104,7 @@
         <v>0.0026660229792492</v>
       </c>
       <c r="AM103" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN103">
         <v>0.0062754689148565</v>
@@ -30278,7 +30275,7 @@
         <v>5608278.16173986</v>
       </c>
       <c r="CS103" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="CT103">
         <v>-0.8495964311677586</v>
@@ -30376,7 +30373,7 @@
         <v>0.0095889911638783</v>
       </c>
       <c r="AM104" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN104">
         <v>0.0276610340172863</v>
@@ -30547,7 +30544,7 @@
         <v>16198187.75410762</v>
       </c>
       <c r="CS104" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="CT104">
         <v>-0.8581350323980486</v>
@@ -30645,7 +30642,7 @@
         <v>0.0090102837599302</v>
       </c>
       <c r="AM105" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN105">
         <v>0.0216087690726687</v>
@@ -30816,7 +30813,7 @@
         <v>10577375.81046865</v>
       </c>
       <c r="CS105" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="CT105">
         <v>-0.8842562871250494</v>
@@ -30914,7 +30911,7 @@
         <v>0.0050995967216395</v>
       </c>
       <c r="AM106" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN106">
         <v>0.0064663828879011</v>
@@ -31085,7 +31082,7 @@
         <v>8161103.390277231</v>
       </c>
       <c r="CS106" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="CT106">
         <v>-0.8751724322696175</v>
@@ -31183,7 +31180,7 @@
         <v>0.008368149950938699</v>
       </c>
       <c r="AM107" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN107">
         <v>0.0044562593205472</v>
@@ -31354,7 +31351,7 @@
         <v>8562542.046147738</v>
       </c>
       <c r="CS107" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="CT107">
         <v>-0.9169005340500024</v>
@@ -31452,7 +31449,7 @@
         <v>0.0065618399294816</v>
       </c>
       <c r="AM108" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN108">
         <v>0.0115970759513037</v>
@@ -31623,7 +31620,7 @@
         <v>5094802.189709073</v>
       </c>
       <c r="CS108" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="CT108">
         <v>-0.807087633056609</v>
@@ -31721,7 +31718,7 @@
         <v>0.0039283848188842</v>
       </c>
       <c r="AM109" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN109">
         <v>0.0506122383924143</v>
@@ -31892,7 +31889,7 @@
         <v>2688942.923710383</v>
       </c>
       <c r="CS109" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="CT109">
         <v>-0.6156032480827009</v>
@@ -31990,7 +31987,7 @@
         <v>0.0110575018573894</v>
       </c>
       <c r="AM110" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN110">
         <v>0.0182408073926103</v>
@@ -32161,7 +32158,7 @@
         <v>7113237.577421894</v>
       </c>
       <c r="CS110" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="CT110">
         <v>-0.7629790982692873</v>
@@ -32259,7 +32256,7 @@
         <v>0.0079211631943229</v>
       </c>
       <c r="AM111" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN111">
         <v>0.0160665598628607</v>
@@ -32430,7 +32427,7 @@
         <v>7296357.590261763</v>
       </c>
       <c r="CS111" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="CT111">
         <v>-0.8942723506201351</v>
@@ -32528,7 +32525,7 @@
         <v>0.0045682228774332</v>
       </c>
       <c r="AM112" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN112">
         <v>0.037886406926907</v>
@@ -32699,7 +32696,7 @@
         <v>646350.5069878154</v>
       </c>
       <c r="CS112" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="CT112">
         <v>-0.0916621825765546</v>
@@ -32797,7 +32794,7 @@
         <v>0.0103540243512939</v>
       </c>
       <c r="AM113" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN113">
         <v>0.0123420077084287</v>
@@ -32968,7 +32965,7 @@
         <v>16980708.42353759</v>
       </c>
       <c r="CS113" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="CT113">
         <v>-0.8006705745635164</v>
@@ -33066,7 +33063,7 @@
         <v>0.0064839021721033</v>
       </c>
       <c r="AM114" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN114">
         <v>0.0163921516174475</v>
@@ -33237,7 +33234,7 @@
         <v>778558.4127862654</v>
       </c>
       <c r="CS114" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="CT114">
         <v>-0.7935423347142916</v>
@@ -33335,7 +33332,7 @@
         <v>0.0115121978063762</v>
       </c>
       <c r="AM115" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN115">
         <v>0.0122833373375532</v>
@@ -33506,7 +33503,7 @@
         <v>22312718.74654885</v>
       </c>
       <c r="CS115" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="CT115">
         <v>-0.833943178203995</v>
@@ -33604,7 +33601,7 @@
         <v>0.0085575638145724</v>
       </c>
       <c r="AM116" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN116">
         <v>0.0253654749054445</v>
@@ -33775,7 +33772,7 @@
         <v>55051148.20247716</v>
       </c>
       <c r="CS116" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="CT116">
         <v>-0.7450076808546802</v>
@@ -33873,7 +33870,7 @@
         <v>0.0073550550024841</v>
       </c>
       <c r="AM117" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN117">
         <v>0.0189839179655455</v>
@@ -34044,7 +34041,7 @@
         <v>7593228.666961946</v>
       </c>
       <c r="CS117" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="CT117">
         <v>-0.5920454049159357</v>
@@ -34142,7 +34139,7 @@
         <v>0.0080994776472478</v>
       </c>
       <c r="AM118" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN118">
         <v>0.0067043103411634</v>
@@ -34313,7 +34310,7 @@
         <v>8613700.914603613</v>
       </c>
       <c r="CS118" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="CT118">
         <v>-0.9326775287918464</v>
@@ -34411,7 +34408,7 @@
         <v>0.0068550971234694</v>
       </c>
       <c r="AM119" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN119">
         <v>0.009392776226783601</v>
@@ -34582,7 +34579,7 @@
         <v>2380328.733367264</v>
       </c>
       <c r="CS119" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="CT119">
         <v>-0.955941339278515</v>
@@ -34680,7 +34677,7 @@
         <v>0.0038610240640448</v>
       </c>
       <c r="AM120" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN120">
         <v>0.0077083561528932</v>
@@ -34851,7 +34848,7 @@
         <v>872704.4135421006</v>
       </c>
       <c r="CS120" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="CT120">
         <v>-0.8980421674690441</v>
@@ -34949,7 +34946,7 @@
         <v>0.007825344507997999</v>
       </c>
       <c r="AM121" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN121">
         <v>0.0327708854210512</v>
@@ -35120,7 +35117,7 @@
         <v>10271258.08902804</v>
       </c>
       <c r="CS121" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="CT121">
         <v>-0.7644558396778582</v>
@@ -35218,7 +35215,7 @@
         <v>0.0053863780237919</v>
       </c>
       <c r="AM122" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN122">
         <v>0.0318217118436193</v>
@@ -35389,7 +35386,7 @@
         <v>4219262.028734344</v>
       </c>
       <c r="CS122" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="CT122">
         <v>-0.7390744315992817</v>
@@ -35487,7 +35484,7 @@
         <v>0.008317099460099901</v>
       </c>
       <c r="AM123" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN123">
         <v>0.0412544366764669</v>
@@ -35658,7 +35655,7 @@
         <v>7884481.26725769</v>
       </c>
       <c r="CS123" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="CT123">
         <v>-0.7831546722232047</v>
@@ -35756,7 +35753,7 @@
         <v>0.0032418393755305</v>
       </c>
       <c r="AM124" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN124">
         <v>0.0499292345312228</v>
@@ -35927,7 +35924,7 @@
         <v>4199685.074142367</v>
       </c>
       <c r="CS124" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="CT124">
         <v>-0.7053510752114568</v>
@@ -36025,7 +36022,7 @@
         <v>0.0105307693727994</v>
       </c>
       <c r="AM125" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN125">
         <v>0.0209369586410007</v>
@@ -36196,7 +36193,7 @@
         <v>14590537.25038491</v>
       </c>
       <c r="CS125" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="CT125">
         <v>-0.7252315072660098</v>
@@ -36294,7 +36291,7 @@
         <v>0.0051130877078413</v>
       </c>
       <c r="AM126" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN126">
         <v>0.0123868401976321</v>
@@ -36465,7 +36462,7 @@
         <v>716228.3326648935</v>
       </c>
       <c r="CS126" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="CT126">
         <v>-0.892232561911074</v>
@@ -36563,7 +36560,7 @@
         <v>0.0103267254619839</v>
       </c>
       <c r="AM127" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN127">
         <v>0.0276741525944277</v>
@@ -36734,7 +36731,7 @@
         <v>7960049.437302528</v>
       </c>
       <c r="CS127" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="CT127">
         <v>-0.7368411844597273</v>
@@ -36832,7 +36829,7 @@
         <v>0.001129927884937</v>
       </c>
       <c r="AM128" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN128">
         <v>0.0069498164483821</v>
@@ -37003,7 +37000,7 @@
         <v>1259981.153790825</v>
       </c>
       <c r="CS128" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="CT128">
         <v>-0.9143802706411296</v>
@@ -37101,7 +37098,7 @@
         <v>0.0097288328816258</v>
       </c>
       <c r="AM129" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN129">
         <v>0.0275626982729415</v>
@@ -37272,7 +37269,7 @@
         <v>16803825.65057263</v>
       </c>
       <c r="CS129" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="CT129">
         <v>-0.8590793790924167</v>
@@ -37370,7 +37367,7 @@
         <v>0.0115638527937927</v>
       </c>
       <c r="AM130" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN130">
         <v>0.009514899377222301</v>
@@ -37541,7 +37538,7 @@
         <v>7461415.917733567</v>
       </c>
       <c r="CS130" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="CT130">
         <v>-0.7834455371012616</v>
@@ -37639,7 +37636,7 @@
         <v>0.0066617897392062</v>
       </c>
       <c r="AM131" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN131">
         <v>0.0175240810959318</v>
@@ -37810,7 +37807,7 @@
         <v>1295517.443775632</v>
       </c>
       <c r="CS131" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="CT131">
         <v>-0.7832286955751367</v>
@@ -37908,7 +37905,7 @@
         <v>0.0073511543785546</v>
       </c>
       <c r="AM132" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN132">
         <v>0.0171480510071521</v>
@@ -38079,7 +38076,7 @@
         <v>7436893.530962305</v>
       </c>
       <c r="CS132" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="CT132">
         <v>-0.8091587172086132</v>
@@ -38177,7 +38174,7 @@
         <v>0.0033730418087468</v>
       </c>
       <c r="AM133" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN133">
         <v>0.009616489085314</v>
@@ -38348,7 +38345,7 @@
         <v>867003.1587181734</v>
       </c>
       <c r="CS133" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="CT133">
         <v>-0.9000180936758766</v>
@@ -38446,7 +38443,7 @@
         <v>0.0074087938346481</v>
       </c>
       <c r="AM134" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN134">
         <v>0.0409391807131387</v>
@@ -38617,7 +38614,7 @@
         <v>3390202.150984915</v>
       </c>
       <c r="CS134" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="CT134">
         <v>-0.6893066803315582</v>
@@ -38715,7 +38712,7 @@
         <v>0.0083849241650579</v>
       </c>
       <c r="AM135" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN135">
         <v>0.0422126511911422</v>
@@ -38886,7 +38883,7 @@
         <v>8715912.703511165</v>
       </c>
       <c r="CS135" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="CT135">
         <v>-0.8034449984146571</v>
@@ -38984,7 +38981,7 @@
         <v>0.008401051909799701</v>
       </c>
       <c r="AM136" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN136">
         <v>0.020710590359547</v>
@@ -39155,7 +39152,7 @@
         <v>15549669.36335931</v>
       </c>
       <c r="CS136" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="CT136">
         <v>-0.8182238609422743</v>
@@ -39253,7 +39250,7 @@
         <v>0.0077330551594838</v>
       </c>
       <c r="AM137" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN137">
         <v>0.0190728510027463</v>
@@ -39424,7 +39421,7 @@
         <v>8185952.559251163</v>
       </c>
       <c r="CS137" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="CT137">
         <v>-0.8729982178980289</v>
@@ -39522,7 +39519,7 @@
         <v>0.010898810531027</v>
       </c>
       <c r="AM138" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN138">
         <v>0.035028448432581</v>
@@ -39693,7 +39690,7 @@
         <v>1792741.222718281</v>
       </c>
       <c r="CS138" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="CT138">
         <v>-0.7176955593761354</v>
@@ -39791,7 +39788,7 @@
         <v>0.0049947080562063</v>
       </c>
       <c r="AM139" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN139">
         <v>0.0090224491293264</v>
@@ -39962,7 +39959,7 @@
         <v>4157882.239708048</v>
       </c>
       <c r="CS139" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="CT139">
         <v>-0.8723102032515645</v>
@@ -40060,7 +40057,7 @@
         <v>0.006652001977027</v>
       </c>
       <c r="AM140" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN140">
         <v>0.0486790527459496</v>
@@ -40231,7 +40228,7 @@
         <v>7172478.294001529</v>
       </c>
       <c r="CS140" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="CT140">
         <v>-0.5365809810110987</v>
@@ -40329,7 +40326,7 @@
         <v>0.009892196288343501</v>
       </c>
       <c r="AM141" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN141">
         <v>0.0262045792935156</v>
@@ -40500,7 +40497,7 @@
         <v>10598803.27492217</v>
       </c>
       <c r="CS141" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="CT141">
         <v>-0.8043091815774359</v>
@@ -40598,7 +40595,7 @@
         <v>0.0032840087191214</v>
       </c>
       <c r="AM142" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN142">
         <v>0.011024599092909</v>
@@ -40769,7 +40766,7 @@
         <v>1954441.87495541</v>
       </c>
       <c r="CS142" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="CT142">
         <v>-0.892071333585829</v>
@@ -40867,7 +40864,7 @@
         <v>0.0042924384175561</v>
       </c>
       <c r="AM143" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN143">
         <v>0.0289399933126468</v>
@@ -41038,7 +41035,7 @@
         <v>2325567.261086872</v>
       </c>
       <c r="CS143" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="CT143">
         <v>-0.7586823863673019</v>
@@ -41136,7 +41133,7 @@
         <v>0.0066499576490462</v>
       </c>
       <c r="AM144" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN144">
         <v>0.0173750820094196</v>
@@ -41307,7 +41304,7 @@
         <v>17826610.98082536</v>
       </c>
       <c r="CS144" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="CT144">
         <v>-0.9111405881388872</v>
@@ -41405,7 +41402,7 @@
         <v>0.0095523432691301</v>
       </c>
       <c r="AM145" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN145">
         <v>0.0220904013262179</v>
@@ -41576,7 +41573,7 @@
         <v>2190979.247087742</v>
       </c>
       <c r="CS145" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="CT145">
         <v>-0.6948709396994353</v>
@@ -41587,169 +41584,169 @@
     </row>
     <row r="146" spans="10:99">
       <c r="J146" t="s">
-        <v>218</v>
+        <v>179</v>
       </c>
       <c r="K146">
-        <v>0.0008094317552731489</v>
+        <v>0.0003006612920797291</v>
       </c>
       <c r="L146">
-        <v>0.0008094317552731489</v>
+        <v>0.0003006612920797291</v>
       </c>
       <c r="M146">
-        <v>0.001294822366811887</v>
+        <v>0.0006591669288791291</v>
       </c>
       <c r="N146">
-        <v>0.001294822366811887</v>
+        <v>0.0006591669288791291</v>
       </c>
       <c r="O146">
-        <v>0.0005767048112779616</v>
+        <v>0.0002176926223928621</v>
       </c>
       <c r="P146">
-        <v>0.0005767048112779616</v>
+        <v>0.0002176926223928621</v>
       </c>
       <c r="Q146">
-        <v>0.00120888913965449</v>
+        <v>0.0003502939601996768</v>
       </c>
       <c r="R146">
-        <v>0.00120888913965449</v>
+        <v>0.0003502939601996768</v>
       </c>
       <c r="S146">
-        <v>4.841526157870145</v>
+        <v>13.16459603066747</v>
       </c>
       <c r="T146">
-        <v>6.846162658534984</v>
+        <v>7.693062975562284</v>
       </c>
       <c r="U146">
-        <v>0.9999821673828903</v>
+        <v>0.9897407973481741</v>
       </c>
       <c r="V146">
-        <v>0.6938615539287721</v>
+        <v>0.6031995381483243</v>
       </c>
       <c r="W146">
-        <v>0.09497469485232257</v>
+        <v>0.0985844511792402</v>
       </c>
       <c r="X146">
-        <v>0.09532047899887716</v>
+        <v>0.07164953255583889</v>
       </c>
       <c r="Y146">
-        <v>0.1815870507556402</v>
+        <v>0.1787176555983328</v>
       </c>
       <c r="Z146">
-        <v>0.1830389294384759</v>
+        <v>0.247566315508007</v>
       </c>
       <c r="AA146">
-        <v>0.9982502254349325</v>
+        <v>0.9951633728963677</v>
       </c>
       <c r="AB146">
-        <v>0.845039733510092</v>
+        <v>0.8362868615300257</v>
       </c>
       <c r="AC146">
-        <v>0.8473503841789751</v>
+        <v>0.7792750654766251</v>
       </c>
       <c r="AD146">
-        <v>0.997041559012992</v>
+        <v>0.9989322028897368</v>
       </c>
       <c r="AE146">
-        <v>0.8219640867968683</v>
+        <v>0.827874478675387</v>
       </c>
       <c r="AF146">
-        <v>0.8192674511295908</v>
+        <v>0.7525001143463156</v>
       </c>
       <c r="AG146">
-        <v>0.009989217099203185</v>
+        <v>0.01198603197666941</v>
       </c>
       <c r="AH146">
-        <v>0.0112725621549946</v>
+        <v>0.008639063327642879</v>
       </c>
       <c r="AI146">
-        <v>0.9982502254349325</v>
+        <v>0.9951633728963677</v>
       </c>
       <c r="AJ146">
-        <v>0.997041559012992</v>
+        <v>0.9989322028897368</v>
       </c>
       <c r="AK146">
-        <v>0.009989217099203185</v>
+        <v>0.01198603197666941</v>
       </c>
       <c r="AL146">
-        <v>0.0112725621549946</v>
+        <v>0.008639063327642879</v>
       </c>
       <c r="AM146" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AN146">
-        <v>0.0629290509487791</v>
+        <v>0.08613291272584166</v>
       </c>
       <c r="AO146">
-        <v>0.1099278580867054</v>
+        <v>0.0329583400133444</v>
       </c>
       <c r="AP146">
-        <v>-328.144462052</v>
+        <v>-2074.048755046</v>
       </c>
       <c r="AQ146">
-        <v>-924.445771572</v>
+        <v>-647.8914794660001</v>
       </c>
       <c r="AR146">
-        <v>23941.36112794793</v>
+        <v>15417.01644128642</v>
       </c>
       <c r="AS146">
-        <v>40398.50998842795</v>
+        <v>25828.327430534</v>
       </c>
       <c r="AT146">
-        <v>23528.18729794793</v>
+        <v>15033.30116495395</v>
       </c>
       <c r="AU146">
-        <v>40398.50998842795</v>
+        <v>25828.235900534</v>
       </c>
       <c r="AV146">
-        <v>1.394136112794793</v>
+        <v>0.5417016441286417</v>
       </c>
       <c r="AW146">
-        <v>3.039850998842795</v>
+        <v>1.5828327430534</v>
       </c>
       <c r="AX146">
-        <v>4.958057310613313</v>
+        <v>1.82313427586692</v>
       </c>
       <c r="AY146">
-        <v>3.501660799711165</v>
+        <v>3.119626252595468</v>
       </c>
       <c r="AZ146">
-        <v>86.81666666666666</v>
+        <v>32.8</v>
       </c>
       <c r="BA146">
-        <v>67.06666666666666</v>
+        <v>73.01666666666667</v>
       </c>
       <c r="BB146">
-        <v>0.06186892398015462</v>
+        <v>0.4319164385691229</v>
       </c>
       <c r="BC146">
-        <v>0.09043022241805039</v>
+        <v>0.01456601041944519</v>
       </c>
       <c r="BD146">
-        <v>-941.0614136434657</v>
+        <v>-5695.48992500237</v>
       </c>
       <c r="BE146">
-        <v>-3114.155643668963</v>
+        <v>-243.5401851911677</v>
       </c>
       <c r="BF146">
-        <v>2271</v>
+        <v>9773</v>
       </c>
       <c r="BG146">
-        <v>1979</v>
+        <v>4349</v>
       </c>
       <c r="BH146">
-        <v>1078.998611111111</v>
+        <v>1439.998611111111</v>
       </c>
       <c r="BI146">
-        <v>2953</v>
+        <v>9184</v>
       </c>
       <c r="BJ146">
-        <v>5408</v>
+        <v>6729</v>
       </c>
       <c r="BK146">
-        <v>5224</v>
+        <v>18957</v>
       </c>
       <c r="BL146">
-        <v>7387</v>
+        <v>11078</v>
       </c>
       <c r="BM146">
         <v>0</v>
@@ -41758,10 +41755,10 @@
         <v>0</v>
       </c>
       <c r="BO146">
-        <v>124</v>
+        <v>8425</v>
       </c>
       <c r="BP146">
-        <v>642</v>
+        <v>3316</v>
       </c>
       <c r="BQ146">
         <v>0</v>
@@ -41770,895 +41767,88 @@
         <v>0</v>
       </c>
       <c r="BS146">
-        <v>2147</v>
+        <v>1348</v>
       </c>
       <c r="BT146">
-        <v>1337</v>
+        <v>1033</v>
       </c>
       <c r="BU146">
-        <v>2953</v>
+        <v>9184</v>
       </c>
       <c r="BV146">
-        <v>5408</v>
+        <v>6729</v>
       </c>
       <c r="BW146">
-        <v>13941.361127948</v>
+        <v>5417.016441286465</v>
       </c>
       <c r="BX146">
-        <v>30398.50998842799</v>
+        <v>15828.32743053398</v>
       </c>
       <c r="BY146">
-        <v>0.09684272780836405</v>
+        <v>0.3728941624432304</v>
       </c>
       <c r="BZ146">
-        <v>0.08451264915172059</v>
+        <v>0.07165386440760954</v>
       </c>
       <c r="CA146">
-        <v>0.2165962201773096</v>
+        <v>1.014621544581806</v>
       </c>
       <c r="CB146">
-        <v>0.18651172313106</v>
+        <v>0.1983944106742799</v>
       </c>
       <c r="CC146">
-        <v>0.01472926243037753</v>
+        <v>0.04576790431830397</v>
       </c>
       <c r="CD146">
-        <v>0.01461622224821496</v>
+        <v>0.01279942344858218</v>
       </c>
       <c r="CE146">
-        <v>0.01570227684644577</v>
+        <v>0.05748299881381747</v>
       </c>
       <c r="CF146">
-        <v>0.01526609143152732</v>
+        <v>0.01265155534126093</v>
       </c>
       <c r="CG146">
-        <v>14269.50559</v>
+        <v>7491.065196332465</v>
       </c>
       <c r="CH146">
-        <v>31322.95575999999</v>
+        <v>16476.21890999998</v>
       </c>
       <c r="CI146">
-        <v>15210.56700364346</v>
+        <v>13186.55512133484</v>
       </c>
       <c r="CJ146">
-        <v>34437.11140366895</v>
+        <v>16719.75909519114</v>
       </c>
       <c r="CK146">
-        <v>0.078977494752154</v>
+        <v>0.04076236855169546</v>
       </c>
       <c r="CL146">
-        <v>0.1240573810034337</v>
+        <v>0.08258268410478285</v>
       </c>
       <c r="CM146">
         <v>10000</v>
       </c>
       <c r="CO146">
-        <v>0.0261420241726841</v>
+        <v>0.003964005671132201</v>
       </c>
       <c r="CP146">
-        <v>0.02262810364134842</v>
+        <v>0.009779809611990395</v>
       </c>
       <c r="CQ146">
-        <v>7572973.222541307</v>
+        <v>7844228.25996128</v>
       </c>
       <c r="CR146">
-        <v>26540564.03326802</v>
+        <v>9465215.444138013</v>
       </c>
       <c r="CS146" s="2">
-        <v>45510.16924547155</v>
+        <v>45510.84732993069</v>
       </c>
       <c r="CT146">
-        <v>-0.7357080524995973</v>
+        <v>-0.8125236089659099</v>
       </c>
       <c r="CU146">
-        <v>-0.6822914041817671</v>
-      </c>
-    </row>
-    <row r="147" spans="10:99">
-      <c r="J147" t="s">
-        <v>238</v>
-      </c>
-      <c r="K147">
-        <v>0.0009271508706103493</v>
-      </c>
-      <c r="L147">
-        <v>0.0009271508706103493</v>
-      </c>
-      <c r="M147">
-        <v>0.0003772496124334612</v>
-      </c>
-      <c r="N147">
-        <v>0.0003772496124334612</v>
-      </c>
-      <c r="O147">
-        <v>0.0007341407739547501</v>
-      </c>
-      <c r="P147">
-        <v>0.0007341407739547501</v>
-      </c>
-      <c r="Q147">
-        <v>0.000427802544585143</v>
-      </c>
-      <c r="R147">
-        <v>0.000427802544585143</v>
-      </c>
-      <c r="S147">
-        <v>5.186290271715415</v>
-      </c>
-      <c r="T147">
-        <v>4.126047943115981</v>
-      </c>
-      <c r="U147">
-        <v>0.9943079530884374</v>
-      </c>
-      <c r="V147">
-        <v>0.7441713851721259</v>
-      </c>
-      <c r="W147">
-        <v>0.08782631912769941</v>
-      </c>
-      <c r="X147">
-        <v>0.09612852812434385</v>
-      </c>
-      <c r="Y147">
-        <v>0.1487338338096725</v>
-      </c>
-      <c r="Z147">
-        <v>0.1765393432169604</v>
-      </c>
-      <c r="AA147">
-        <v>0.9979090421403467</v>
-      </c>
-      <c r="AB147">
-        <v>0.8631748366243617</v>
-      </c>
-      <c r="AC147">
-        <v>0.85245390722169</v>
-      </c>
-      <c r="AD147">
-        <v>0.9973853483851801</v>
-      </c>
-      <c r="AE147">
-        <v>0.8577699950051938</v>
-      </c>
-      <c r="AF147">
-        <v>0.8334553258441252</v>
-      </c>
-      <c r="AG147">
-        <v>0.009891723442382157</v>
-      </c>
-      <c r="AH147">
-        <v>0.01075541834616141</v>
-      </c>
-      <c r="AI147">
-        <v>0.9979090421403467</v>
-      </c>
-      <c r="AJ147">
-        <v>0.9973853483851801</v>
-      </c>
-      <c r="AK147">
-        <v>0.009891723442382157</v>
-      </c>
-      <c r="AL147">
-        <v>0.01075541834616141</v>
-      </c>
-      <c r="AM147" t="s">
-        <v>244</v>
-      </c>
-      <c r="AN147">
-        <v>0.07466532002742356</v>
-      </c>
-      <c r="AO147">
-        <v>0.05158437131730968</v>
-      </c>
-      <c r="AP147">
-        <v>-559.644700872</v>
-      </c>
-      <c r="AQ147">
-        <v>-137.17975723</v>
-      </c>
-      <c r="AR147">
-        <v>27180.94354516747</v>
-      </c>
-      <c r="AS147">
-        <v>15022.66619276996</v>
-      </c>
-      <c r="AT147">
-        <v>25765.66907912802</v>
-      </c>
-      <c r="AU147">
-        <v>15022.66619276996</v>
-      </c>
-      <c r="AV147">
-        <v>1.718094354516747</v>
-      </c>
-      <c r="AW147">
-        <v>0.5022666192769965</v>
-      </c>
-      <c r="AX147">
-        <v>4.626705391718796</v>
-      </c>
-      <c r="AY147">
-        <v>5.805036321425896</v>
-      </c>
-      <c r="AZ147">
-        <v>83.15000000000001</v>
-      </c>
-      <c r="BA147">
-        <v>85.53333333333333</v>
-      </c>
-      <c r="BB147">
-        <v>0.06073549320104688</v>
-      </c>
-      <c r="BC147">
-        <v>0.1979569492821935</v>
-      </c>
-      <c r="BD147">
-        <v>-1147.156492128083</v>
-      </c>
-      <c r="BE147">
-        <v>-1273.531841107445</v>
-      </c>
-      <c r="BF147">
-        <v>2784</v>
-      </c>
-      <c r="BG147">
-        <v>2470</v>
-      </c>
-      <c r="BH147">
-        <v>1078.998611111111</v>
-      </c>
-      <c r="BI147">
-        <v>2812</v>
-      </c>
-      <c r="BJ147">
-        <v>1982</v>
-      </c>
-      <c r="BK147">
-        <v>5596</v>
-      </c>
-      <c r="BL147">
-        <v>4452</v>
-      </c>
-      <c r="BM147">
-        <v>0</v>
-      </c>
-      <c r="BN147">
-        <v>0</v>
-      </c>
-      <c r="BO147">
-        <v>95</v>
-      </c>
-      <c r="BP147">
-        <v>21</v>
-      </c>
-      <c r="BQ147">
-        <v>0</v>
-      </c>
-      <c r="BR147">
-        <v>0</v>
-      </c>
-      <c r="BS147">
-        <v>2689</v>
-      </c>
-      <c r="BT147">
-        <v>2449</v>
-      </c>
-      <c r="BU147">
-        <v>2812</v>
-      </c>
-      <c r="BV147">
-        <v>1982</v>
-      </c>
-      <c r="BW147">
-        <v>17180.94354516744</v>
-      </c>
-      <c r="BX147">
-        <v>5022.666192769993</v>
-      </c>
-      <c r="BY147">
-        <v>0.08872882728817136</v>
-      </c>
-      <c r="BZ147">
-        <v>0.2027142729554022</v>
-      </c>
-      <c r="CA147">
-        <v>0.1658107791868395</v>
-      </c>
-      <c r="CB147">
-        <v>0.3059584933131804</v>
-      </c>
-      <c r="CC147">
-        <v>0.01331063120855579</v>
-      </c>
-      <c r="CD147">
-        <v>0.0240731126461369</v>
-      </c>
-      <c r="CE147">
-        <v>0.01515624390504481</v>
-      </c>
-      <c r="CF147">
-        <v>0.03418969224219068</v>
-      </c>
-      <c r="CG147">
-        <v>17740.58824603944</v>
-      </c>
-      <c r="CH147">
-        <v>5159.845949999994</v>
-      </c>
-      <c r="CI147">
-        <v>18887.74473816753</v>
-      </c>
-      <c r="CJ147">
-        <v>6433.377791107439</v>
-      </c>
-      <c r="CK147">
-        <v>0.09383586056299457</v>
-      </c>
-      <c r="CL147">
-        <v>0.05546030914566657</v>
-      </c>
-      <c r="CM147">
-        <v>10000</v>
-      </c>
-      <c r="CO147">
-        <v>0.03147082673668765</v>
-      </c>
-      <c r="CP147">
-        <v>0.00459512684866973</v>
-      </c>
-      <c r="CQ147">
-        <v>9932751.742502673</v>
-      </c>
-      <c r="CR147">
-        <v>3613938.735498667</v>
-      </c>
-      <c r="CS147" s="2">
-        <v>45510.29086814423</v>
-      </c>
-      <c r="CT147">
-        <v>-0.7509273913693356</v>
-      </c>
-      <c r="CU147">
-        <v>-0.8707969045725891</v>
-      </c>
-    </row>
-    <row r="148" spans="10:99">
-      <c r="J148" t="s">
-        <v>243</v>
-      </c>
-      <c r="K148">
-        <v>0.0008654450215017651</v>
-      </c>
-      <c r="L148">
-        <v>0.0008654450215017651</v>
-      </c>
-      <c r="M148">
-        <v>0.001646773835179527</v>
-      </c>
-      <c r="N148">
-        <v>0.001646773835179527</v>
-      </c>
-      <c r="O148">
-        <v>0.000991580787808899</v>
-      </c>
-      <c r="P148">
-        <v>0.000991580787808899</v>
-      </c>
-      <c r="Q148">
-        <v>0.001622732092626267</v>
-      </c>
-      <c r="R148">
-        <v>0.001622732092626267</v>
-      </c>
-      <c r="S148">
-        <v>8.983329450274754</v>
-      </c>
-      <c r="T148">
-        <v>8.249315530475144</v>
-      </c>
-      <c r="U148">
-        <v>0.9968107850618261</v>
-      </c>
-      <c r="V148">
-        <v>0.7091371326613198</v>
-      </c>
-      <c r="W148">
-        <v>0.08667258536559605</v>
-      </c>
-      <c r="X148">
-        <v>0.09793083597655818</v>
-      </c>
-      <c r="Y148">
-        <v>0.1890133841354915</v>
-      </c>
-      <c r="Z148">
-        <v>0.1721872846152441</v>
-      </c>
-      <c r="AA148">
-        <v>0.9985647018895669</v>
-      </c>
-      <c r="AB148">
-        <v>0.8351064625512248</v>
-      </c>
-      <c r="AC148">
-        <v>0.8646336939548427</v>
-      </c>
-      <c r="AD148">
-        <v>0.9967725907021084</v>
-      </c>
-      <c r="AE148">
-        <v>0.7992347746600847</v>
-      </c>
-      <c r="AF148">
-        <v>0.8298217557593828</v>
-      </c>
-      <c r="AG148">
-        <v>0.008743105624871524</v>
-      </c>
-      <c r="AH148">
-        <v>0.01216711024741432</v>
-      </c>
-      <c r="AI148">
-        <v>0.9985647018895669</v>
-      </c>
-      <c r="AJ148">
-        <v>0.9967725907021084</v>
-      </c>
-      <c r="AK148">
-        <v>0.008743105624871524</v>
-      </c>
-      <c r="AL148">
-        <v>0.01216711024741432</v>
-      </c>
-      <c r="AM148" t="s">
-        <v>244</v>
-      </c>
-      <c r="AN148">
-        <v>0.05947531493518945</v>
-      </c>
-      <c r="AO148">
-        <v>0.1274247914799327</v>
-      </c>
-      <c r="AP148">
-        <v>-551.7531234728001</v>
-      </c>
-      <c r="AQ148">
-        <v>-1961.6248515388</v>
-      </c>
-      <c r="AR148">
-        <v>25431.6692905271</v>
-      </c>
-      <c r="AS148">
-        <v>59026.72629646108</v>
-      </c>
-      <c r="AT148">
-        <v>25422.5117785271</v>
-      </c>
-      <c r="AU148">
-        <v>59026.72629646108</v>
-      </c>
-      <c r="AV148">
-        <v>1.543166929052711</v>
-      </c>
-      <c r="AW148">
-        <v>4.902672629646108</v>
-      </c>
-      <c r="AX148">
-        <v>2.671505709175953</v>
-      </c>
-      <c r="AY148">
-        <v>2.90958052434457</v>
-      </c>
-      <c r="AZ148">
-        <v>34.4</v>
-      </c>
-      <c r="BA148">
-        <v>38.53333333333333</v>
-      </c>
-      <c r="BB148">
-        <v>0.1031095913503279</v>
-      </c>
-      <c r="BC148">
-        <v>0.099712223438205</v>
-      </c>
-      <c r="BD148">
-        <v>-1837.508950473058</v>
-      </c>
-      <c r="BE148">
-        <v>-5647.263013868165</v>
-      </c>
-      <c r="BF148">
-        <v>2956</v>
-      </c>
-      <c r="BG148">
-        <v>4781</v>
-      </c>
-      <c r="BH148">
-        <v>1078.998611111111</v>
-      </c>
-      <c r="BI148">
-        <v>6737</v>
-      </c>
-      <c r="BJ148">
-        <v>4120</v>
-      </c>
-      <c r="BK148">
-        <v>9693</v>
-      </c>
-      <c r="BL148">
-        <v>8901</v>
-      </c>
-      <c r="BM148">
-        <v>0</v>
-      </c>
-      <c r="BN148">
-        <v>0</v>
-      </c>
-      <c r="BO148">
-        <v>128</v>
-      </c>
-      <c r="BP148">
-        <v>755</v>
-      </c>
-      <c r="BQ148">
-        <v>0</v>
-      </c>
-      <c r="BR148">
-        <v>0</v>
-      </c>
-      <c r="BS148">
-        <v>2828</v>
-      </c>
-      <c r="BT148">
-        <v>4026</v>
-      </c>
-      <c r="BU148">
-        <v>6737</v>
-      </c>
-      <c r="BV148">
-        <v>4120</v>
-      </c>
-      <c r="BW148">
-        <v>15431.66929052719</v>
-      </c>
-      <c r="BX148">
-        <v>49026.72629646119</v>
-      </c>
-      <c r="BY148">
-        <v>0.08907029222474379</v>
-      </c>
-      <c r="BZ148">
-        <v>0.08411163445231325</v>
-      </c>
-      <c r="CA148">
-        <v>0.2978207476223507</v>
-      </c>
-      <c r="CB148">
-        <v>0.1454284746387412</v>
-      </c>
-      <c r="CC148">
-        <v>0.01092990615565577</v>
-      </c>
-      <c r="CD148">
-        <v>0.01228844639671559</v>
-      </c>
-      <c r="CE148">
-        <v>0.0124999169776432</v>
-      </c>
-      <c r="CF148">
-        <v>0.01357124514220625</v>
-      </c>
-      <c r="CG148">
-        <v>15983.42241399999</v>
-      </c>
-      <c r="CH148">
-        <v>50988.35114799999</v>
-      </c>
-      <c r="CI148">
-        <v>17820.93136447304</v>
-      </c>
-      <c r="CJ148">
-        <v>56635.61416186816</v>
-      </c>
-      <c r="CK148">
-        <v>0.0897616575121067</v>
-      </c>
-      <c r="CL148">
-        <v>0.1179391706666686</v>
-      </c>
-      <c r="CM148">
-        <v>10000</v>
-      </c>
-      <c r="CO148">
-        <v>0.01463489979534309</v>
-      </c>
-      <c r="CP148">
-        <v>0.05116422751670078</v>
-      </c>
-      <c r="CQ148">
-        <v>22617300.28614038</v>
-      </c>
-      <c r="CR148">
-        <v>33517948.77339607</v>
-      </c>
-      <c r="CS148" s="2">
-        <v>45510.50511107766</v>
-      </c>
-      <c r="CT148">
-        <v>-0.7516800885976392</v>
-      </c>
-      <c r="CU148">
-        <v>-0.552387130925049</v>
-      </c>
-    </row>
-    <row r="149" spans="10:99">
-      <c r="J149" t="s">
-        <v>239</v>
-      </c>
-      <c r="K149">
-        <v>0.001539670459458575</v>
-      </c>
-      <c r="L149">
-        <v>0.001539670459458575</v>
-      </c>
-      <c r="M149">
-        <v>0.000967767001506914</v>
-      </c>
-      <c r="N149">
-        <v>0.000967767001506914</v>
-      </c>
-      <c r="O149">
-        <v>0.001528178840837024</v>
-      </c>
-      <c r="P149">
-        <v>0.001528178840837024</v>
-      </c>
-      <c r="Q149">
-        <v>0.0008568539482927795</v>
-      </c>
-      <c r="R149">
-        <v>0.0008568539482927795</v>
-      </c>
-      <c r="S149">
-        <v>25.55543558417511</v>
-      </c>
-      <c r="T149">
-        <v>10.43389564174606</v>
-      </c>
-      <c r="U149">
-        <v>0.9903830827773132</v>
-      </c>
-      <c r="V149">
-        <v>0.6983167081863534</v>
-      </c>
-      <c r="W149">
-        <v>0.07767822502634231</v>
-      </c>
-      <c r="X149">
-        <v>0.07619329814793283</v>
-      </c>
-      <c r="Y149">
-        <v>0.2265564135738889</v>
-      </c>
-      <c r="Z149">
-        <v>0.177853027024439</v>
-      </c>
-      <c r="AA149">
-        <v>0.9983501622472053</v>
-      </c>
-      <c r="AB149">
-        <v>0.8566234782846035</v>
-      </c>
-      <c r="AC149">
-        <v>0.8380233689002388</v>
-      </c>
-      <c r="AD149">
-        <v>0.9982271555000344</v>
-      </c>
-      <c r="AE149">
-        <v>0.7736909263770486</v>
-      </c>
-      <c r="AF149">
-        <v>0.8223674871415904</v>
-      </c>
-      <c r="AG149">
-        <v>0.00863693076930128</v>
-      </c>
-      <c r="AH149">
-        <v>0.008640155143380991</v>
-      </c>
-      <c r="AI149">
-        <v>0.9983501622472053</v>
-      </c>
-      <c r="AJ149">
-        <v>0.9982271555000344</v>
-      </c>
-      <c r="AK149">
-        <v>0.00863693076930128</v>
-      </c>
-      <c r="AL149">
-        <v>0.008640155143380991</v>
-      </c>
-      <c r="AM149" t="s">
-        <v>244</v>
-      </c>
-      <c r="AN149">
-        <v>0.07371412979936612</v>
-      </c>
-      <c r="AO149">
-        <v>0.05717297154639175</v>
-      </c>
-      <c r="AP149">
-        <v>-1856.69298268</v>
-      </c>
-      <c r="AQ149">
-        <v>-483.25193874</v>
-      </c>
-      <c r="AR149">
-        <v>40356.99241732022</v>
-      </c>
-      <c r="AS149">
-        <v>24041.51726126008</v>
-      </c>
-      <c r="AT149">
-        <v>40355.13961732022</v>
-      </c>
-      <c r="AU149">
-        <v>24038.10026126008</v>
-      </c>
-      <c r="AV149">
-        <v>3.035699241732022</v>
-      </c>
-      <c r="AW149">
-        <v>1.404151726126007</v>
-      </c>
-      <c r="AX149">
-        <v>0.9391509162567245</v>
-      </c>
-      <c r="AY149">
-        <v>2.300007046471479</v>
-      </c>
-      <c r="AZ149">
-        <v>37.93333333333333</v>
-      </c>
-      <c r="BA149">
-        <v>41.28333333333333</v>
-      </c>
-      <c r="BB149">
-        <v>0.07609453288998462</v>
-      </c>
-      <c r="BC149">
-        <v>0.07532181822408669</v>
-      </c>
-      <c r="BD149">
-        <v>-2653.177657715952</v>
-      </c>
-      <c r="BE149">
-        <v>-1183.148956027105</v>
-      </c>
-      <c r="BF149">
-        <v>7830</v>
-      </c>
-      <c r="BG149">
-        <v>5405</v>
-      </c>
-      <c r="BH149">
-        <v>906.8520833333333</v>
-      </c>
-      <c r="BI149">
-        <v>15345</v>
-      </c>
-      <c r="BJ149">
-        <v>4057</v>
-      </c>
-      <c r="BK149">
-        <v>23175</v>
-      </c>
-      <c r="BL149">
-        <v>9462</v>
-      </c>
-      <c r="BM149">
-        <v>0</v>
-      </c>
-      <c r="BN149">
-        <v>0</v>
-      </c>
-      <c r="BO149">
-        <v>3750</v>
-      </c>
-      <c r="BP149">
-        <v>732</v>
-      </c>
-      <c r="BQ149">
-        <v>0</v>
-      </c>
-      <c r="BR149">
-        <v>0</v>
-      </c>
-      <c r="BS149">
-        <v>4080</v>
-      </c>
-      <c r="BT149">
-        <v>4673</v>
-      </c>
-      <c r="BU149">
-        <v>15345</v>
-      </c>
-      <c r="BV149">
-        <v>4057</v>
-      </c>
-      <c r="BW149">
-        <v>30356.99241731995</v>
-      </c>
-      <c r="BX149">
-        <v>14041.51726126001</v>
-      </c>
-      <c r="BY149">
-        <v>0.07944929949855256</v>
-      </c>
-      <c r="BZ149">
-        <v>0.07290428891734235</v>
-      </c>
-      <c r="CA149">
-        <v>0.2939414045616529</v>
-      </c>
-      <c r="CB149">
-        <v>0.1508373732980492</v>
-      </c>
-      <c r="CC149">
-        <v>0.008541457371382059</v>
-      </c>
-      <c r="CD149">
-        <v>0.01502445815399398</v>
-      </c>
-      <c r="CE149">
-        <v>0.01132079572183098</v>
-      </c>
-      <c r="CF149">
-        <v>0.01358610203418608</v>
-      </c>
-      <c r="CG149">
-        <v>32213.68539999995</v>
-      </c>
-      <c r="CH149">
-        <v>14524.76920000001</v>
-      </c>
-      <c r="CI149">
-        <v>34866.8630577159</v>
-      </c>
-      <c r="CJ149">
-        <v>15707.91815602711</v>
-      </c>
-      <c r="CK149">
-        <v>0.1826593380074046</v>
-      </c>
-      <c r="CL149">
-        <v>0.09736031104338029</v>
-      </c>
-      <c r="CM149">
-        <v>10000</v>
-      </c>
-      <c r="CO149">
-        <v>0.03349260314251585</v>
-      </c>
-      <c r="CP149">
-        <v>0.01741247817697326</v>
-      </c>
-      <c r="CQ149">
-        <v>58107883.34426937</v>
-      </c>
-      <c r="CR149">
-        <v>9758740.845571002</v>
-      </c>
-      <c r="CS149" s="2">
-        <v>45510.63778221698</v>
-      </c>
-      <c r="CT149">
-        <v>-0.7358834399820444</v>
-      </c>
-      <c r="CU149">
-        <v>-0.7141006607483422</v>
+        <v>-0.8391421413768273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update KSMUSDT.json at 2024-08-07_05-33-50 bestfile_scores 0.0008034584150236224 bestfile_sharp 0.11426319667372078
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="387">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1536,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU146"/>
+  <dimension ref="A1:CU147"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -41849,6 +41849,275 @@
       </c>
       <c r="CU146">
         <v>-0.8391421413768273</v>
+      </c>
+    </row>
+    <row r="147" spans="10:99">
+      <c r="J147" t="s">
+        <v>201</v>
+      </c>
+      <c r="K147">
+        <v>0.000854942508918155</v>
+      </c>
+      <c r="L147">
+        <v>0.000854942508918155</v>
+      </c>
+      <c r="M147">
+        <v>0.0004317584820443532</v>
+      </c>
+      <c r="N147">
+        <v>0.0004317584820443532</v>
+      </c>
+      <c r="O147">
+        <v>0.0006125857001524126</v>
+      </c>
+      <c r="P147">
+        <v>0.0006125857001524126</v>
+      </c>
+      <c r="Q147">
+        <v>0.0002983100812595119</v>
+      </c>
+      <c r="R147">
+        <v>0.0002983100812595119</v>
+      </c>
+      <c r="S147">
+        <v>8.813897389947329</v>
+      </c>
+      <c r="T147">
+        <v>29.6819730728907</v>
+      </c>
+      <c r="U147">
+        <v>0.9908295496065532</v>
+      </c>
+      <c r="V147">
+        <v>0.835211186003199</v>
+      </c>
+      <c r="W147">
+        <v>0.09019879698108996</v>
+      </c>
+      <c r="X147">
+        <v>0.03590977280826664</v>
+      </c>
+      <c r="Y147">
+        <v>0.2432050215665514</v>
+      </c>
+      <c r="Z147">
+        <v>0.09574965133783017</v>
+      </c>
+      <c r="AA147">
+        <v>0.9986031239756389</v>
+      </c>
+      <c r="AB147">
+        <v>0.7798737296227506</v>
+      </c>
+      <c r="AC147">
+        <v>0.9195447367252673</v>
+      </c>
+      <c r="AD147">
+        <v>0.9994916294275633</v>
+      </c>
+      <c r="AE147">
+        <v>0.7582436254230526</v>
+      </c>
+      <c r="AF147">
+        <v>0.9102088890419561</v>
+      </c>
+      <c r="AG147">
+        <v>0.009903730347895115</v>
+      </c>
+      <c r="AH147">
+        <v>0.003881457052144715</v>
+      </c>
+      <c r="AI147">
+        <v>0.9986031239756389</v>
+      </c>
+      <c r="AJ147">
+        <v>0.9994916294275633</v>
+      </c>
+      <c r="AK147">
+        <v>0.009903730347895115</v>
+      </c>
+      <c r="AL147">
+        <v>0.003881457052144715</v>
+      </c>
+      <c r="AM147" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN147">
+        <v>0.04621057237520097</v>
+      </c>
+      <c r="AO147">
+        <v>0.02646859110361865</v>
+      </c>
+      <c r="AP147">
+        <v>-1298.767165448</v>
+      </c>
+      <c r="AQ147">
+        <v>-1876.229917604</v>
+      </c>
+      <c r="AR147">
+        <v>34232.48857455169</v>
+      </c>
+      <c r="AS147">
+        <v>18618.99930050792</v>
+      </c>
+      <c r="AT147">
+        <v>34232.48857455169</v>
+      </c>
+      <c r="AU147">
+        <v>18619.31066050792</v>
+      </c>
+      <c r="AV147">
+        <v>2.42324885745517</v>
+      </c>
+      <c r="AW147">
+        <v>0.8618999300507917</v>
+      </c>
+      <c r="AX147">
+        <v>2.722869224910041</v>
+      </c>
+      <c r="AY147">
+        <v>0.8085901125383121</v>
+      </c>
+      <c r="AZ147">
+        <v>61.43333333333333</v>
+      </c>
+      <c r="BA147">
+        <v>110.9666666666667</v>
+      </c>
+      <c r="BB147">
+        <v>0.09249180583421727</v>
+      </c>
+      <c r="BC147">
+        <v>0.05758358994526326</v>
+      </c>
+      <c r="BD147">
+        <v>-2602.105373581276</v>
+      </c>
+      <c r="BE147">
+        <v>-641.307513765596</v>
+      </c>
+      <c r="BF147">
+        <v>4533</v>
+      </c>
+      <c r="BG147">
+        <v>17288</v>
+      </c>
+      <c r="BH147">
+        <v>1439.998611111111</v>
+      </c>
+      <c r="BI147">
+        <v>8159</v>
+      </c>
+      <c r="BJ147">
+        <v>25454</v>
+      </c>
+      <c r="BK147">
+        <v>12692</v>
+      </c>
+      <c r="BL147">
+        <v>42742</v>
+      </c>
+      <c r="BM147">
+        <v>0</v>
+      </c>
+      <c r="BN147">
+        <v>0</v>
+      </c>
+      <c r="BO147">
+        <v>3466</v>
+      </c>
+      <c r="BP147">
+        <v>16479</v>
+      </c>
+      <c r="BQ147">
+        <v>0</v>
+      </c>
+      <c r="BR147">
+        <v>0</v>
+      </c>
+      <c r="BS147">
+        <v>1067</v>
+      </c>
+      <c r="BT147">
+        <v>809</v>
+      </c>
+      <c r="BU147">
+        <v>8159</v>
+      </c>
+      <c r="BV147">
+        <v>25454</v>
+      </c>
+      <c r="BW147">
+        <v>24232.48857455198</v>
+      </c>
+      <c r="BX147">
+        <v>8619.446462395941</v>
+      </c>
+      <c r="BY147">
+        <v>0.0969668546792643</v>
+      </c>
+      <c r="BZ147">
+        <v>0.0364228070630991</v>
+      </c>
+      <c r="CA147">
+        <v>0.3174017098814577</v>
+      </c>
+      <c r="CB147">
+        <v>0.08239266961537647</v>
+      </c>
+      <c r="CC147">
+        <v>0.01100354317540885</v>
+      </c>
+      <c r="CD147">
+        <v>0.007859398996726275</v>
+      </c>
+      <c r="CE147">
+        <v>0.01637250283452613</v>
+      </c>
+      <c r="CF147">
+        <v>0.007120688634382433</v>
+      </c>
+      <c r="CG147">
+        <v>25531.25573999998</v>
+      </c>
+      <c r="CH147">
+        <v>10495.67637999994</v>
+      </c>
+      <c r="CI147">
+        <v>28133.36111358125</v>
+      </c>
+      <c r="CJ147">
+        <v>11136.98389376554</v>
+      </c>
+      <c r="CK147">
+        <v>0.09974444233706491</v>
+      </c>
+      <c r="CL147">
+        <v>0.09157175948218245</v>
+      </c>
+      <c r="CM147">
+        <v>10000</v>
+      </c>
+      <c r="CO147">
+        <v>0.02239518532449871</v>
+      </c>
+      <c r="CP147">
+        <v>0.009866612655883799</v>
+      </c>
+      <c r="CQ147">
+        <v>21824015.57534306</v>
+      </c>
+      <c r="CR147">
+        <v>18938191.45644107</v>
+      </c>
+      <c r="CS147" s="2">
+        <v>45511.0311169706</v>
+      </c>
+      <c r="CT147">
+        <v>-0.7908510809186831</v>
+      </c>
+      <c r="CU147">
+        <v>-0.9173245807835106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update THETAUSDT.json at 2024-08-07_14-54-31 bestfile_scores 0.0009506474001933885 bestfile_sharp 0.08103309864754131
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="387">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1536,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU147"/>
+  <dimension ref="A1:CU149"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -42118,6 +42118,544 @@
       </c>
       <c r="CU147">
         <v>-0.9173245807835106</v>
+      </c>
+    </row>
+    <row r="148" spans="10:99">
+      <c r="J148" t="s">
+        <v>190</v>
+      </c>
+      <c r="K148">
+        <v>0.0007607554171973341</v>
+      </c>
+      <c r="L148">
+        <v>0.0007607554171973341</v>
+      </c>
+      <c r="M148">
+        <v>0.0009812366869994538</v>
+      </c>
+      <c r="N148">
+        <v>0.0009812366869994538</v>
+      </c>
+      <c r="O148">
+        <v>0.0006323790460851742</v>
+      </c>
+      <c r="P148">
+        <v>0.0006323790460851742</v>
+      </c>
+      <c r="Q148">
+        <v>0.0008394625098125275</v>
+      </c>
+      <c r="R148">
+        <v>0.0008394625098125275</v>
+      </c>
+      <c r="S148">
+        <v>6.772977628391993</v>
+      </c>
+      <c r="T148">
+        <v>13.74283578618982</v>
+      </c>
+      <c r="U148">
+        <v>0.9917077405534929</v>
+      </c>
+      <c r="V148">
+        <v>0.6483165740397461</v>
+      </c>
+      <c r="W148">
+        <v>0.02894093353884385</v>
+      </c>
+      <c r="X148">
+        <v>0.09393990372129114</v>
+      </c>
+      <c r="Y148">
+        <v>0.2154420984790889</v>
+      </c>
+      <c r="Z148">
+        <v>0.223628205597902</v>
+      </c>
+      <c r="AA148">
+        <v>0.9994772706874676</v>
+      </c>
+      <c r="AB148">
+        <v>0.8421914763435698</v>
+      </c>
+      <c r="AC148">
+        <v>0.8194564353021796</v>
+      </c>
+      <c r="AD148">
+        <v>0.997653318823376</v>
+      </c>
+      <c r="AE148">
+        <v>0.7890782216754897</v>
+      </c>
+      <c r="AF148">
+        <v>0.7834648854683399</v>
+      </c>
+      <c r="AG148">
+        <v>0.004034387758639863</v>
+      </c>
+      <c r="AH148">
+        <v>0.010802890795369</v>
+      </c>
+      <c r="AI148">
+        <v>0.9994772706874676</v>
+      </c>
+      <c r="AJ148">
+        <v>0.997653318823376</v>
+      </c>
+      <c r="AK148">
+        <v>0.004034387758639863</v>
+      </c>
+      <c r="AL148">
+        <v>0.010802890795369</v>
+      </c>
+      <c r="AM148" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN148">
+        <v>0.02355574948693454</v>
+      </c>
+      <c r="AO148">
+        <v>0.07775347061663966</v>
+      </c>
+      <c r="AP148">
+        <v>-492.97480768</v>
+      </c>
+      <c r="AQ148">
+        <v>-1527.60816546</v>
+      </c>
+      <c r="AR148">
+        <v>28816.01099231987</v>
+      </c>
+      <c r="AS148">
+        <v>39154.2689345401</v>
+      </c>
+      <c r="AT148">
+        <v>28816.26719231987</v>
+      </c>
+      <c r="AU148">
+        <v>39156.1233345401</v>
+      </c>
+      <c r="AV148">
+        <v>1.881601099231987</v>
+      </c>
+      <c r="AW148">
+        <v>2.91542689345401</v>
+      </c>
+      <c r="AX148">
+        <v>3.543824933687003</v>
+      </c>
+      <c r="AY148">
+        <v>1.74636862745098</v>
+      </c>
+      <c r="AZ148">
+        <v>88.31666666666666</v>
+      </c>
+      <c r="BA148">
+        <v>79.86666666666666</v>
+      </c>
+      <c r="BB148">
+        <v>0.04727097251029871</v>
+      </c>
+      <c r="BC148">
+        <v>0.0530361645528751</v>
+      </c>
+      <c r="BD148">
+        <v>-958.042119655489</v>
+      </c>
+      <c r="BE148">
+        <v>-1718.385667704362</v>
+      </c>
+      <c r="BF148">
+        <v>3539</v>
+      </c>
+      <c r="BG148">
+        <v>5200</v>
+      </c>
+      <c r="BH148">
+        <v>1391.706944444444</v>
+      </c>
+      <c r="BI148">
+        <v>5887</v>
+      </c>
+      <c r="BJ148">
+        <v>13926</v>
+      </c>
+      <c r="BK148">
+        <v>9426</v>
+      </c>
+      <c r="BL148">
+        <v>19126</v>
+      </c>
+      <c r="BM148">
+        <v>0</v>
+      </c>
+      <c r="BN148">
+        <v>0</v>
+      </c>
+      <c r="BO148">
+        <v>220</v>
+      </c>
+      <c r="BP148">
+        <v>3348</v>
+      </c>
+      <c r="BQ148">
+        <v>0</v>
+      </c>
+      <c r="BR148">
+        <v>0</v>
+      </c>
+      <c r="BS148">
+        <v>3319</v>
+      </c>
+      <c r="BT148">
+        <v>1852</v>
+      </c>
+      <c r="BU148">
+        <v>5887</v>
+      </c>
+      <c r="BV148">
+        <v>13926</v>
+      </c>
+      <c r="BW148">
+        <v>18816.01099231996</v>
+      </c>
+      <c r="BX148">
+        <v>29154.26893454001</v>
+      </c>
+      <c r="BY148">
+        <v>0.06037443910645804</v>
+      </c>
+      <c r="BZ148">
+        <v>0.0808934247240536</v>
+      </c>
+      <c r="CA148">
+        <v>0.4830253043819779</v>
+      </c>
+      <c r="CB148">
+        <v>0.1791826362818437</v>
+      </c>
+      <c r="CC148">
+        <v>0.01546386176285824</v>
+      </c>
+      <c r="CD148">
+        <v>0.01275030211096267</v>
+      </c>
+      <c r="CE148">
+        <v>0.01375738409307254</v>
+      </c>
+      <c r="CF148">
+        <v>0.01479921692285975</v>
+      </c>
+      <c r="CG148">
+        <v>19308.98579999996</v>
+      </c>
+      <c r="CH148">
+        <v>30681.87710000001</v>
+      </c>
+      <c r="CI148">
+        <v>20267.02791965545</v>
+      </c>
+      <c r="CJ148">
+        <v>32400.26276770437</v>
+      </c>
+      <c r="CK148">
+        <v>0.1142631966737208</v>
+      </c>
+      <c r="CL148">
+        <v>0.09193550622721315</v>
+      </c>
+      <c r="CM148">
+        <v>10000</v>
+      </c>
+      <c r="CO148">
+        <v>0.002484881144841626</v>
+      </c>
+      <c r="CP148">
+        <v>0.03344111131069996</v>
+      </c>
+      <c r="CQ148">
+        <v>16376196.08893238</v>
+      </c>
+      <c r="CR148">
+        <v>43044880.09408081</v>
+      </c>
+      <c r="CS148" s="2">
+        <v>45511.23185884381</v>
+      </c>
+      <c r="CT148">
+        <v>-0.8743035118239124</v>
+      </c>
+      <c r="CU148">
+        <v>-0.6887529826640726</v>
+      </c>
+    </row>
+    <row r="149" spans="10:99">
+      <c r="J149" t="s">
+        <v>206</v>
+      </c>
+      <c r="K149">
+        <v>0.001479499085291547</v>
+      </c>
+      <c r="L149">
+        <v>0.001479499085291547</v>
+      </c>
+      <c r="M149">
+        <v>0.0003726094215379394</v>
+      </c>
+      <c r="N149">
+        <v>0.0003726094215379394</v>
+      </c>
+      <c r="O149">
+        <v>0.001041931768115267</v>
+      </c>
+      <c r="P149">
+        <v>0.001041931768115267</v>
+      </c>
+      <c r="Q149">
+        <v>0.0002769132258935159</v>
+      </c>
+      <c r="R149">
+        <v>0.0002769132258935159</v>
+      </c>
+      <c r="S149">
+        <v>7.29342905815236</v>
+      </c>
+      <c r="T149">
+        <v>3.226644735645823</v>
+      </c>
+      <c r="U149">
+        <v>0.9951659576093447</v>
+      </c>
+      <c r="V149">
+        <v>0.9937438575106513</v>
+      </c>
+      <c r="W149">
+        <v>0.09855207867442294</v>
+      </c>
+      <c r="X149">
+        <v>0.0425988230748508</v>
+      </c>
+      <c r="Y149">
+        <v>0.2414096178825358</v>
+      </c>
+      <c r="Z149">
+        <v>0.1569911322184733</v>
+      </c>
+      <c r="AA149">
+        <v>0.9979579662872851</v>
+      </c>
+      <c r="AB149">
+        <v>0.7919176251971737</v>
+      </c>
+      <c r="AC149">
+        <v>0.8814342437072773</v>
+      </c>
+      <c r="AD149">
+        <v>0.9990411550355666</v>
+      </c>
+      <c r="AE149">
+        <v>0.6421151682005247</v>
+      </c>
+      <c r="AF149">
+        <v>0.8434549178201648</v>
+      </c>
+      <c r="AG149">
+        <v>0.01098554071611368</v>
+      </c>
+      <c r="AH149">
+        <v>0.004959918010916282</v>
+      </c>
+      <c r="AI149">
+        <v>0.9979579662872851</v>
+      </c>
+      <c r="AJ149">
+        <v>0.9990411550355666</v>
+      </c>
+      <c r="AK149">
+        <v>0.01098554071611368</v>
+      </c>
+      <c r="AL149">
+        <v>0.004959918010916282</v>
+      </c>
+      <c r="AM149" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN149">
+        <v>0.0632697333701665</v>
+      </c>
+      <c r="AO149">
+        <v>0.02356369953032022</v>
+      </c>
+      <c r="AP149">
+        <v>-1874.943362112</v>
+      </c>
+      <c r="AQ149">
+        <v>-161.929665476</v>
+      </c>
+      <c r="AR149">
+        <v>72149.78691587639</v>
+      </c>
+      <c r="AS149">
+        <v>16453.74103452402</v>
+      </c>
+      <c r="AT149">
+        <v>70952.21419788794</v>
+      </c>
+      <c r="AU149">
+        <v>16455.64727452402</v>
+      </c>
+      <c r="AV149">
+        <v>6.214978691587639</v>
+      </c>
+      <c r="AW149">
+        <v>0.6453741034524016</v>
+      </c>
+      <c r="AX149">
+        <v>3.290651073724525</v>
+      </c>
+      <c r="AY149">
+        <v>7.438729128014843</v>
+      </c>
+      <c r="AZ149">
+        <v>99.83333333333333</v>
+      </c>
+      <c r="BA149">
+        <v>21.63333333333333</v>
+      </c>
+      <c r="BB149">
+        <v>0.06617616443045932</v>
+      </c>
+      <c r="BC149">
+        <v>0.3322728638795527</v>
+      </c>
+      <c r="BD149">
+        <v>-4537.1631319604</v>
+      </c>
+      <c r="BE149">
+        <v>-3292.075057402672</v>
+      </c>
+      <c r="BF149">
+        <v>4441</v>
+      </c>
+      <c r="BG149">
+        <v>2200</v>
+      </c>
+      <c r="BH149">
+        <v>1336.682638888889</v>
+      </c>
+      <c r="BI149">
+        <v>5308</v>
+      </c>
+      <c r="BJ149">
+        <v>2113</v>
+      </c>
+      <c r="BK149">
+        <v>9749</v>
+      </c>
+      <c r="BL149">
+        <v>4313</v>
+      </c>
+      <c r="BM149">
+        <v>0</v>
+      </c>
+      <c r="BN149">
+        <v>0</v>
+      </c>
+      <c r="BO149">
+        <v>217</v>
+      </c>
+      <c r="BP149">
+        <v>640</v>
+      </c>
+      <c r="BQ149">
+        <v>0</v>
+      </c>
+      <c r="BR149">
+        <v>0</v>
+      </c>
+      <c r="BS149">
+        <v>4224</v>
+      </c>
+      <c r="BT149">
+        <v>1560</v>
+      </c>
+      <c r="BU149">
+        <v>5308</v>
+      </c>
+      <c r="BV149">
+        <v>2113</v>
+      </c>
+      <c r="BW149">
+        <v>62149.78691587646</v>
+      </c>
+      <c r="BX149">
+        <v>6453.741034523994</v>
+      </c>
+      <c r="BY149">
+        <v>0.1121990440240032</v>
+      </c>
+      <c r="BZ149">
+        <v>0.1393015359259272</v>
+      </c>
+      <c r="CA149">
+        <v>0.3473978273728501</v>
+      </c>
+      <c r="CB149">
+        <v>0.2045643542854885</v>
+      </c>
+      <c r="CC149">
+        <v>0.01832148890560509</v>
+      </c>
+      <c r="CD149">
+        <v>0.02573074330113078</v>
+      </c>
+      <c r="CE149">
+        <v>0.01959512440507218</v>
+      </c>
+      <c r="CF149">
+        <v>0.02521356073813698</v>
+      </c>
+      <c r="CG149">
+        <v>64024.73027798846</v>
+      </c>
+      <c r="CH149">
+        <v>6615.670699999994</v>
+      </c>
+      <c r="CI149">
+        <v>68561.89340994885</v>
+      </c>
+      <c r="CJ149">
+        <v>9907.745757402667</v>
+      </c>
+      <c r="CK149">
+        <v>0.112504700057311</v>
+      </c>
+      <c r="CL149">
+        <v>0.06284556911514147</v>
+      </c>
+      <c r="CM149">
+        <v>10000</v>
+      </c>
+      <c r="CO149">
+        <v>0.01776697213390686</v>
+      </c>
+      <c r="CP149">
+        <v>0</v>
+      </c>
+      <c r="CQ149">
+        <v>39426472.20941308</v>
+      </c>
+      <c r="CR149">
+        <v>1497091.069727402</v>
+      </c>
+      <c r="CS149" s="2">
+        <v>45511.42653623307</v>
+      </c>
+      <c r="CT149">
+        <v>-0.6490041422520464</v>
+      </c>
+      <c r="CU149">
+        <v>-0.8959799270302342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update DYDXUSDT.json at 2024-08-07_18-11-41 bestfile_scores 0.0009318630504310643 bestfile_sharp 0.15299940942250698
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis_clock.xlsx
+++ b/optimized/logs/analysis_clock.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="387">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1536,7 +1536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU149"/>
+  <dimension ref="A1:CU150"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -42656,6 +42656,275 @@
       </c>
       <c r="CU149">
         <v>-0.8959799270302342</v>
+      </c>
+    </row>
+    <row r="150" spans="10:99">
+      <c r="J150" t="s">
+        <v>202</v>
+      </c>
+      <c r="K150">
+        <v>0.0008009736526357614</v>
+      </c>
+      <c r="L150">
+        <v>0.0008009736526357614</v>
+      </c>
+      <c r="M150">
+        <v>0.001117110144327249</v>
+      </c>
+      <c r="N150">
+        <v>0.001117110144327249</v>
+      </c>
+      <c r="O150">
+        <v>0.0007668097814315766</v>
+      </c>
+      <c r="P150">
+        <v>0.0007668097814315766</v>
+      </c>
+      <c r="Q150">
+        <v>0.001117696022378967</v>
+      </c>
+      <c r="R150">
+        <v>0.001117696022378967</v>
+      </c>
+      <c r="S150">
+        <v>6.039589158554358</v>
+      </c>
+      <c r="T150">
+        <v>28.84377782000175</v>
+      </c>
+      <c r="U150">
+        <v>0.9999801418105023</v>
+      </c>
+      <c r="V150">
+        <v>0.6102809819071024</v>
+      </c>
+      <c r="W150">
+        <v>0.09953249263962105</v>
+      </c>
+      <c r="X150">
+        <v>0.0915233933548991</v>
+      </c>
+      <c r="Y150">
+        <v>0.2395449107841185</v>
+      </c>
+      <c r="Z150">
+        <v>0.2465246021956368</v>
+      </c>
+      <c r="AA150">
+        <v>0.9974263935268729</v>
+      </c>
+      <c r="AB150">
+        <v>0.7790926908234403</v>
+      </c>
+      <c r="AC150">
+        <v>0.8212224357907854</v>
+      </c>
+      <c r="AD150">
+        <v>0.9978560510725616</v>
+      </c>
+      <c r="AE150">
+        <v>0.7610708058892569</v>
+      </c>
+      <c r="AF150">
+        <v>0.7579905289721663</v>
+      </c>
+      <c r="AG150">
+        <v>0.01164652268898005</v>
+      </c>
+      <c r="AH150">
+        <v>0.009911220052056382</v>
+      </c>
+      <c r="AI150">
+        <v>0.9974263935268729</v>
+      </c>
+      <c r="AJ150">
+        <v>0.9978560510725616</v>
+      </c>
+      <c r="AK150">
+        <v>0.01164652268898005</v>
+      </c>
+      <c r="AL150">
+        <v>0.009911220052056382</v>
+      </c>
+      <c r="AM150" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN150">
+        <v>0.07356089259561639</v>
+      </c>
+      <c r="AO150">
+        <v>0.08339590988074361</v>
+      </c>
+      <c r="AP150">
+        <v>-463.6832376020001</v>
+      </c>
+      <c r="AQ150">
+        <v>-4058.094557976</v>
+      </c>
+      <c r="AR150">
+        <v>31674.8935323979</v>
+      </c>
+      <c r="AS150">
+        <v>49915.137102024</v>
+      </c>
+      <c r="AT150">
+        <v>31675.7481323979</v>
+      </c>
+      <c r="AU150">
+        <v>49915.137102024</v>
+      </c>
+      <c r="AV150">
+        <v>2.16748935323979</v>
+      </c>
+      <c r="AW150">
+        <v>3.991513710202399</v>
+      </c>
+      <c r="AX150">
+        <v>3.974191199018706</v>
+      </c>
+      <c r="AY150">
+        <v>0.8320524550167734</v>
+      </c>
+      <c r="AZ150">
+        <v>53.81666666666667</v>
+      </c>
+      <c r="BA150">
+        <v>48.08333333333334</v>
+      </c>
+      <c r="BB150">
+        <v>0.06639372580466396</v>
+      </c>
+      <c r="BC150">
+        <v>0.07655850907524696</v>
+      </c>
+      <c r="BD150">
+        <v>-1574.392371173534</v>
+      </c>
+      <c r="BE150">
+        <v>-3645.628974001092</v>
+      </c>
+      <c r="BF150">
+        <v>5561</v>
+      </c>
+      <c r="BG150">
+        <v>16088</v>
+      </c>
+      <c r="BH150">
+        <v>1439.998611111111</v>
+      </c>
+      <c r="BI150">
+        <v>3136</v>
+      </c>
+      <c r="BJ150">
+        <v>25447</v>
+      </c>
+      <c r="BK150">
+        <v>8697</v>
+      </c>
+      <c r="BL150">
+        <v>41535</v>
+      </c>
+      <c r="BM150">
+        <v>0</v>
+      </c>
+      <c r="BN150">
+        <v>0</v>
+      </c>
+      <c r="BO150">
+        <v>119</v>
+      </c>
+      <c r="BP150">
+        <v>13867</v>
+      </c>
+      <c r="BQ150">
+        <v>0</v>
+      </c>
+      <c r="BR150">
+        <v>0</v>
+      </c>
+      <c r="BS150">
+        <v>5442</v>
+      </c>
+      <c r="BT150">
+        <v>2221</v>
+      </c>
+      <c r="BU150">
+        <v>3136</v>
+      </c>
+      <c r="BV150">
+        <v>25447</v>
+      </c>
+      <c r="BW150">
+        <v>21674.893532398</v>
+      </c>
+      <c r="BX150">
+        <v>39915.13710202399</v>
+      </c>
+      <c r="BY150">
+        <v>0.1256437453875369</v>
+      </c>
+      <c r="BZ150">
+        <v>0.07959396596750523</v>
+      </c>
+      <c r="CA150">
+        <v>0.3181106583163244</v>
+      </c>
+      <c r="CB150">
+        <v>0.1948491069010549</v>
+      </c>
+      <c r="CC150">
+        <v>0.02187197466246163</v>
+      </c>
+      <c r="CD150">
+        <v>0.01130770938117127</v>
+      </c>
+      <c r="CE150">
+        <v>0.02242199299679752</v>
+      </c>
+      <c r="CF150">
+        <v>0.01213956748712042</v>
+      </c>
+      <c r="CG150">
+        <v>22138.57677</v>
+      </c>
+      <c r="CH150">
+        <v>43973.23165999999</v>
+      </c>
+      <c r="CI150">
+        <v>23712.96914117353</v>
+      </c>
+      <c r="CJ150">
+        <v>47618.86063400108</v>
+      </c>
+      <c r="CK150">
+        <v>0.08103309864754131</v>
+      </c>
+      <c r="CL150">
+        <v>0.1224613625078401</v>
+      </c>
+      <c r="CM150">
+        <v>10000</v>
+      </c>
+      <c r="CO150">
+        <v>0.01993576574751888</v>
+      </c>
+      <c r="CP150">
+        <v>0.0261855849078441</v>
+      </c>
+      <c r="CQ150">
+        <v>15112790.32983612</v>
+      </c>
+      <c r="CR150">
+        <v>64371731.63863062</v>
+      </c>
+      <c r="CS150" s="2">
+        <v>45511.62121535985</v>
+      </c>
+      <c r="CT150">
+        <v>-0.7649046647376796</v>
+      </c>
+      <c r="CU150">
+        <v>-0.7475799015843646</v>
       </c>
     </row>
   </sheetData>

</xml_diff>